<commit_message>
new updates on data processing engine
</commit_message>
<xml_diff>
--- a/P012-excavator-split_data_files/output/01_06_07_2017_template.xlsx
+++ b/P012-excavator-split_data_files/output/01_06_07_2017_template.xlsx
@@ -3,15 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6945" yWindow="2085" windowWidth="20490" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excavator" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MPDM 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MPDM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Excavator'!$A$1:$S$111</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'MPDM 1'!$A$1:$T$120</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'MPDM'!$A$1:$T$120</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" concurrentCalc="0"/>
 </workbook>
@@ -56,10 +56,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="8"/>
     </font>
   </fonts>
@@ -343,12 +345,12 @@
     </border>
   </borders>
   <cellStyleXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
@@ -470,11 +472,11 @@
     <xf numFmtId="9" fontId="3" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="43" fontId="3" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="43" fontId="3" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -494,6 +496,15 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -504,19 +515,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -525,9 +524,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -991,31 +987,31 @@
         </is>
       </c>
       <c r="C6" s="10" t="n"/>
-      <c r="D6" s="11" t="n"/>
+      <c r="D6" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
           <t>Number of Equipment Types:</t>
         </is>
       </c>
-      <c r="H6" s="57" t="n"/>
+      <c r="H6" s="56" t="n"/>
       <c r="I6" s="48" t="n"/>
-      <c r="J6" s="2" t="n"/>
+      <c r="J6" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="L6" s="47" t="inlineStr">
         <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
           <t>06_07_2017</t>
         </is>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>Yared Girma</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
     </row>
     <row r="7" ht="27" customHeight="1"/>
     <row r="8" ht="15" customHeight="1" thickBot="1">
@@ -1030,92 +1026,92 @@
       <c r="O8" s="5" t="n"/>
     </row>
     <row r="9" ht="32.25" customHeight="1" thickBot="1">
-      <c r="B9" s="58" t="inlineStr">
+      <c r="B9" s="57" t="inlineStr">
         <is>
           <t>Equipment Tag</t>
         </is>
       </c>
-      <c r="C9" s="58" t="inlineStr">
+      <c r="C9" s="57" t="inlineStr">
         <is>
           <t>Manpower (Foreman, Operator, Helper, Laborers, etc.)</t>
         </is>
       </c>
-      <c r="D9" s="58" t="inlineStr">
+      <c r="D9" s="57" t="inlineStr">
         <is>
           <t>Excavator Type (Face Shovel, Hoe, Loader)</t>
         </is>
       </c>
-      <c r="E9" s="58" t="inlineStr">
+      <c r="E9" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">Task Type </t>
         </is>
       </c>
-      <c r="F9" s="58" t="inlineStr">
+      <c r="F9" s="57" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G9" s="58" t="inlineStr">
+      <c r="G9" s="57" t="inlineStr">
         <is>
           <t>Soil Type</t>
         </is>
       </c>
-      <c r="H9" s="58" t="inlineStr">
+      <c r="H9" s="57" t="inlineStr">
         <is>
           <t>Factors</t>
         </is>
       </c>
-      <c r="I9" s="59" t="n"/>
-      <c r="J9" s="59" t="n"/>
-      <c r="K9" s="57" t="n"/>
-      <c r="L9" s="58" t="inlineStr">
+      <c r="I9" s="58" t="n"/>
+      <c r="J9" s="58" t="n"/>
+      <c r="K9" s="56" t="n"/>
+      <c r="L9" s="57" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="M9" s="58" t="inlineStr">
+      <c r="M9" s="57" t="inlineStr">
         <is>
           <t>Q Heaped Bucket Capcity</t>
         </is>
       </c>
-      <c r="N9" s="58" t="inlineStr">
+      <c r="N9" s="57" t="inlineStr">
         <is>
           <t>T Cycle Time (seconds)</t>
         </is>
       </c>
-      <c r="O9" s="58" t="inlineStr">
+      <c r="O9" s="57" t="inlineStr">
         <is>
           <t>Productivity (m3/hr)</t>
         </is>
       </c>
-      <c r="P9" s="58" t="inlineStr">
+      <c r="P9" s="57" t="inlineStr">
         <is>
           <t>Ideal Productivity (m3/hr)</t>
         </is>
       </c>
-      <c r="Q9" s="58" t="inlineStr">
+      <c r="Q9" s="57" t="inlineStr">
         <is>
           <t>Overall Method Productivity (m3/hr)</t>
         </is>
       </c>
-      <c r="R9" s="58" t="inlineStr">
+      <c r="R9" s="57" t="inlineStr">
         <is>
           <t>Ideal Cycle Variability (%)</t>
         </is>
       </c>
-      <c r="S9" s="58" t="inlineStr">
+      <c r="S9" s="57" t="inlineStr">
         <is>
           <t>Overall Cycle Vairability (%)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42.75" customHeight="1" thickBot="1">
-      <c r="B10" s="60" t="n"/>
-      <c r="C10" s="60" t="n"/>
-      <c r="D10" s="60" t="n"/>
-      <c r="E10" s="60" t="n"/>
-      <c r="F10" s="60" t="n"/>
-      <c r="G10" s="60" t="n"/>
+      <c r="B10" s="59" t="n"/>
+      <c r="C10" s="59" t="n"/>
+      <c r="D10" s="59" t="n"/>
+      <c r="E10" s="59" t="n"/>
+      <c r="F10" s="59" t="n"/>
+      <c r="G10" s="59" t="n"/>
       <c r="H10" s="6" t="inlineStr">
         <is>
           <t>F (Bucket Fill Factor)</t>
@@ -1136,14 +1132,14 @@
           <t xml:space="preserve">Efficiency </t>
         </is>
       </c>
-      <c r="L10" s="60" t="n"/>
-      <c r="M10" s="60" t="n"/>
-      <c r="N10" s="60" t="n"/>
-      <c r="O10" s="60" t="n"/>
-      <c r="P10" s="60" t="n"/>
-      <c r="Q10" s="60" t="n"/>
-      <c r="R10" s="60" t="n"/>
-      <c r="S10" s="60" t="n"/>
+      <c r="L10" s="59" t="n"/>
+      <c r="M10" s="59" t="n"/>
+      <c r="N10" s="59" t="n"/>
+      <c r="O10" s="59" t="n"/>
+      <c r="P10" s="59" t="n"/>
+      <c r="Q10" s="59" t="n"/>
+      <c r="R10" s="59" t="n"/>
+      <c r="S10" s="59" t="n"/>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="B11" s="7" t="n">
@@ -1194,19 +1190,19 @@
         <v/>
       </c>
       <c r="P11" s="39">
-        <f>'MPDM 1'!H118*H11*I11*J11*M11</f>
+        <f>MPDM!H118*H11*I11*J11*M11</f>
         <v/>
       </c>
       <c r="Q11" s="39">
-        <f>'MPDM 1'!K118*H11*I11*J11*M11</f>
+        <f>MPDM!K118*H11*I11*J11*M11</f>
         <v/>
       </c>
       <c r="R11" s="40">
-        <f>'MPDM 1'!H119</f>
+        <f>MPDM!H119</f>
         <v/>
       </c>
       <c r="S11" s="40">
-        <f>'MPDM 1'!K119</f>
+        <f>MPDM!K119</f>
         <v/>
       </c>
     </row>
@@ -6458,16 +6454,16 @@
       <c r="S110" s="9" t="n"/>
     </row>
     <row r="111" customFormat="1" s="5">
-      <c r="B111" s="56" t="inlineStr">
+      <c r="B111" s="49" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="C111" s="61" t="n"/>
-      <c r="D111" s="61" t="n"/>
-      <c r="E111" s="61" t="n"/>
-      <c r="F111" s="61" t="n"/>
-      <c r="G111" s="61" t="n"/>
+      <c r="C111" s="60" t="n"/>
+      <c r="D111" s="60" t="n"/>
+      <c r="E111" s="60" t="n"/>
+      <c r="F111" s="60" t="n"/>
+      <c r="G111" s="60" t="n"/>
       <c r="H111" s="5">
         <f>AVERAGE(H11:H110)</f>
         <v/>
@@ -6509,8 +6505,8 @@
     <mergeCell ref="B2:O2"/>
     <mergeCell ref="S9:S10"/>
     <mergeCell ref="G6:H6"/>
+    <mergeCell ref="B9:B10"/>
     <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B9:B10"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="H9:K9"/>
     <mergeCell ref="L9:L10"/>
@@ -6598,15 +6594,19 @@
           <t>Project Code:</t>
         </is>
       </c>
-      <c r="B6" s="62" t="n"/>
-      <c r="C6" s="57" t="n"/>
+      <c r="B6" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="n"/>
       <c r="F6" s="19" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
       </c>
-      <c r="G6" s="53" t="n">
-        <v>1</v>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>06_07_2017</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="27" customHeight="1" thickBot="1"/>
@@ -6616,14 +6616,14 @@
           <t>Operation/Activity:</t>
         </is>
       </c>
-      <c r="B8" s="62" t="n"/>
-      <c r="C8" s="57" t="n"/>
+      <c r="B8" s="55" t="n"/>
+      <c r="C8" s="2" t="n"/>
       <c r="F8" s="19" t="inlineStr">
         <is>
           <t>Unit of Time:</t>
         </is>
       </c>
-      <c r="G8" s="53" t="inlineStr">
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>Seconds</t>
         </is>
@@ -6635,63 +6635,67 @@
           <t>Equipment Type:</t>
         </is>
       </c>
-      <c r="B9" s="62" t="n"/>
-      <c r="C9" s="57" t="n"/>
+      <c r="B9" s="55" t="inlineStr">
+        <is>
+          <t>excavator</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" thickBot="1">
       <c r="A10" s="20" t="n"/>
       <c r="B10" s="20" t="n"/>
     </row>
     <row r="11" ht="32.25" customHeight="1" thickBot="1">
-      <c r="A11" s="58" t="inlineStr">
+      <c r="A11" s="57" t="inlineStr">
         <is>
           <t>Production Cycle Number</t>
         </is>
       </c>
-      <c r="B11" s="58" t="inlineStr">
+      <c r="B11" s="57" t="inlineStr">
         <is>
           <t>Cycle Time (Seconds)</t>
         </is>
       </c>
-      <c r="C11" s="58" t="inlineStr">
+      <c r="C11" s="57" t="inlineStr">
         <is>
           <t>Delay (Insert Delay us 1 or if more than one delay event a proportion of the delay). Leave zero values as BLANK</t>
         </is>
       </c>
-      <c r="D11" s="59" t="n"/>
-      <c r="E11" s="59" t="n"/>
-      <c r="F11" s="59" t="n"/>
-      <c r="G11" s="59" t="n"/>
-      <c r="H11" s="57" t="n"/>
-      <c r="I11" s="51" t="n"/>
-      <c r="J11" s="51" t="n"/>
-      <c r="K11" s="51" t="n"/>
-      <c r="L11" s="51" t="n"/>
+      <c r="D11" s="58" t="n"/>
+      <c r="E11" s="58" t="n"/>
+      <c r="F11" s="58" t="n"/>
+      <c r="G11" s="58" t="n"/>
+      <c r="H11" s="56" t="n"/>
+      <c r="I11" s="54" t="n"/>
+      <c r="J11" s="54" t="n"/>
+      <c r="K11" s="54" t="n"/>
+      <c r="L11" s="54" t="n"/>
       <c r="M11" s="21" t="n"/>
-      <c r="O11" s="58" t="inlineStr">
+      <c r="O11" s="57" t="inlineStr">
         <is>
           <t>Delay (Time)</t>
         </is>
       </c>
-      <c r="P11" s="59" t="n"/>
-      <c r="Q11" s="59" t="n"/>
-      <c r="R11" s="59" t="n"/>
-      <c r="S11" s="59" t="n"/>
-      <c r="T11" s="57" t="n"/>
-      <c r="V11" s="58" t="inlineStr">
+      <c r="P11" s="58" t="n"/>
+      <c r="Q11" s="58" t="n"/>
+      <c r="R11" s="58" t="n"/>
+      <c r="S11" s="58" t="n"/>
+      <c r="T11" s="56" t="n"/>
+      <c r="V11" s="57" t="inlineStr">
         <is>
           <t>Delay (Time)</t>
         </is>
       </c>
-      <c r="W11" s="59" t="n"/>
-      <c r="X11" s="59" t="n"/>
-      <c r="Y11" s="59" t="n"/>
-      <c r="Z11" s="59" t="n"/>
-      <c r="AA11" s="57" t="n"/>
+      <c r="W11" s="58" t="n"/>
+      <c r="X11" s="58" t="n"/>
+      <c r="Y11" s="58" t="n"/>
+      <c r="Z11" s="58" t="n"/>
+      <c r="AA11" s="56" t="n"/>
     </row>
     <row r="12" ht="42.75" customHeight="1" thickBot="1">
-      <c r="A12" s="60" t="n"/>
-      <c r="B12" s="60" t="n"/>
+      <c r="A12" s="59" t="n"/>
+      <c r="B12" s="59" t="n"/>
       <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Enviroment</t>
@@ -6815,27 +6819,27 @@
       <c r="B13" s="23" t="n">
         <v>19</v>
       </c>
-      <c r="C13" s="54">
+      <c r="C13" s="41">
         <f>IF(SUM($V13:$AA13), ROUND(V13/SUM($V13:$AA13), 2),0)</f>
         <v/>
       </c>
-      <c r="D13" s="54">
+      <c r="D13" s="41">
         <f>IF(SUM($V13:$AA13), ROUND(W13/SUM($V13:$AA13), 2),0)</f>
         <v/>
       </c>
-      <c r="E13" s="54">
+      <c r="E13" s="41">
         <f>IF(SUM($V13:$AA13), ROUND(X13/SUM($V13:$AA13), 2),0)</f>
         <v/>
       </c>
-      <c r="F13" s="54">
+      <c r="F13" s="41">
         <f>IF(SUM($V13:$AA13), ROUND(Y13/SUM($V13:$AA13), 2),0)</f>
         <v/>
       </c>
-      <c r="G13" s="54">
+      <c r="G13" s="41">
         <f>IF(SUM($V13:$AA13), ROUND(Z13/SUM($V13:$AA13), 2),0)</f>
         <v/>
       </c>
-      <c r="H13" s="54">
+      <c r="H13" s="41">
         <f>IF(SUM($V13:$AA13), ROUND(AA13/SUM($V13:$AA13), 2),0)</f>
         <v/>
       </c>
@@ -6897,27 +6901,27 @@
       <c r="B14" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C14" s="54">
+      <c r="C14" s="41">
         <f>IF(SUM($V14:$AA14), ROUND(V14/SUM($V14:$AA14), 2),0)</f>
         <v/>
       </c>
-      <c r="D14" s="54">
+      <c r="D14" s="41">
         <f>IF(SUM($V14:$AA14), ROUND(W14/SUM($V14:$AA14), 2),0)</f>
         <v/>
       </c>
-      <c r="E14" s="54">
+      <c r="E14" s="41">
         <f>IF(SUM($V14:$AA14), ROUND(X14/SUM($V14:$AA14), 2),0)</f>
         <v/>
       </c>
-      <c r="F14" s="54">
+      <c r="F14" s="41">
         <f>IF(SUM($V14:$AA14), ROUND(Y14/SUM($V14:$AA14), 2),0)</f>
         <v/>
       </c>
-      <c r="G14" s="54">
+      <c r="G14" s="41">
         <f>IF(SUM($V14:$AA14), ROUND(Z14/SUM($V14:$AA14), 2),0)</f>
         <v/>
       </c>
-      <c r="H14" s="54">
+      <c r="H14" s="41">
         <f>IF(SUM($V14:$AA14), ROUND(AA14/SUM($V14:$AA14), 2),0)</f>
         <v/>
       </c>
@@ -6979,27 +6983,27 @@
       <c r="B15" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C15" s="54">
+      <c r="C15" s="41">
         <f>IF(SUM($V15:$AA15), ROUND(V15/SUM($V15:$AA15), 2),0)</f>
         <v/>
       </c>
-      <c r="D15" s="54">
+      <c r="D15" s="41">
         <f>IF(SUM($V15:$AA15), ROUND(W15/SUM($V15:$AA15), 2),0)</f>
         <v/>
       </c>
-      <c r="E15" s="54">
+      <c r="E15" s="41">
         <f>IF(SUM($V15:$AA15), ROUND(X15/SUM($V15:$AA15), 2),0)</f>
         <v/>
       </c>
-      <c r="F15" s="54">
+      <c r="F15" s="41">
         <f>IF(SUM($V15:$AA15), ROUND(Y15/SUM($V15:$AA15), 2),0)</f>
         <v/>
       </c>
-      <c r="G15" s="54">
+      <c r="G15" s="41">
         <f>IF(SUM($V15:$AA15), ROUND(Z15/SUM($V15:$AA15), 2),0)</f>
         <v/>
       </c>
-      <c r="H15" s="54">
+      <c r="H15" s="41">
         <f>IF(SUM($V15:$AA15), ROUND(AA15/SUM($V15:$AA15), 2),0)</f>
         <v/>
       </c>
@@ -7061,27 +7065,27 @@
       <c r="B16" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C16" s="54">
+      <c r="C16" s="41">
         <f>IF(SUM($V16:$AA16), ROUND(V16/SUM($V16:$AA16), 2),0)</f>
         <v/>
       </c>
-      <c r="D16" s="54">
+      <c r="D16" s="41">
         <f>IF(SUM($V16:$AA16), ROUND(W16/SUM($V16:$AA16), 2),0)</f>
         <v/>
       </c>
-      <c r="E16" s="54">
+      <c r="E16" s="41">
         <f>IF(SUM($V16:$AA16), ROUND(X16/SUM($V16:$AA16), 2),0)</f>
         <v/>
       </c>
-      <c r="F16" s="54">
+      <c r="F16" s="41">
         <f>IF(SUM($V16:$AA16), ROUND(Y16/SUM($V16:$AA16), 2),0)</f>
         <v/>
       </c>
-      <c r="G16" s="54">
+      <c r="G16" s="41">
         <f>IF(SUM($V16:$AA16), ROUND(Z16/SUM($V16:$AA16), 2),0)</f>
         <v/>
       </c>
-      <c r="H16" s="54">
+      <c r="H16" s="41">
         <f>IF(SUM($V16:$AA16), ROUND(AA16/SUM($V16:$AA16), 2),0)</f>
         <v/>
       </c>
@@ -7143,27 +7147,27 @@
       <c r="B17" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C17" s="54">
+      <c r="C17" s="41">
         <f>IF(SUM($V17:$AA17), ROUND(V17/SUM($V17:$AA17), 2),0)</f>
         <v/>
       </c>
-      <c r="D17" s="54">
+      <c r="D17" s="41">
         <f>IF(SUM($V17:$AA17), ROUND(W17/SUM($V17:$AA17), 2),0)</f>
         <v/>
       </c>
-      <c r="E17" s="54">
+      <c r="E17" s="41">
         <f>IF(SUM($V17:$AA17), ROUND(X17/SUM($V17:$AA17), 2),0)</f>
         <v/>
       </c>
-      <c r="F17" s="54">
+      <c r="F17" s="41">
         <f>IF(SUM($V17:$AA17), ROUND(Y17/SUM($V17:$AA17), 2),0)</f>
         <v/>
       </c>
-      <c r="G17" s="54">
+      <c r="G17" s="41">
         <f>IF(SUM($V17:$AA17), ROUND(Z17/SUM($V17:$AA17), 2),0)</f>
         <v/>
       </c>
-      <c r="H17" s="54">
+      <c r="H17" s="41">
         <f>IF(SUM($V17:$AA17), ROUND(AA17/SUM($V17:$AA17), 2),0)</f>
         <v/>
       </c>
@@ -7225,27 +7229,27 @@
       <c r="B18" s="26" t="n">
         <v>32</v>
       </c>
-      <c r="C18" s="54">
+      <c r="C18" s="41">
         <f>IF(SUM($V18:$AA18), ROUND(V18/SUM($V18:$AA18), 2),0)</f>
         <v/>
       </c>
-      <c r="D18" s="54">
+      <c r="D18" s="41">
         <f>IF(SUM($V18:$AA18), ROUND(W18/SUM($V18:$AA18), 2),0)</f>
         <v/>
       </c>
-      <c r="E18" s="54">
+      <c r="E18" s="41">
         <f>IF(SUM($V18:$AA18), ROUND(X18/SUM($V18:$AA18), 2),0)</f>
         <v/>
       </c>
-      <c r="F18" s="54">
+      <c r="F18" s="41">
         <f>IF(SUM($V18:$AA18), ROUND(Y18/SUM($V18:$AA18), 2),0)</f>
         <v/>
       </c>
-      <c r="G18" s="54">
+      <c r="G18" s="41">
         <f>IF(SUM($V18:$AA18), ROUND(Z18/SUM($V18:$AA18), 2),0)</f>
         <v/>
       </c>
-      <c r="H18" s="54">
+      <c r="H18" s="41">
         <f>IF(SUM($V18:$AA18), ROUND(AA18/SUM($V18:$AA18), 2),0)</f>
         <v/>
       </c>
@@ -7307,27 +7311,27 @@
       <c r="B19" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C19" s="54">
+      <c r="C19" s="41">
         <f>IF(SUM($V19:$AA19), ROUND(V19/SUM($V19:$AA19), 2),0)</f>
         <v/>
       </c>
-      <c r="D19" s="54">
+      <c r="D19" s="41">
         <f>IF(SUM($V19:$AA19), ROUND(W19/SUM($V19:$AA19), 2),0)</f>
         <v/>
       </c>
-      <c r="E19" s="54">
+      <c r="E19" s="41">
         <f>IF(SUM($V19:$AA19), ROUND(X19/SUM($V19:$AA19), 2),0)</f>
         <v/>
       </c>
-      <c r="F19" s="54">
+      <c r="F19" s="41">
         <f>IF(SUM($V19:$AA19), ROUND(Y19/SUM($V19:$AA19), 2),0)</f>
         <v/>
       </c>
-      <c r="G19" s="54">
+      <c r="G19" s="41">
         <f>IF(SUM($V19:$AA19), ROUND(Z19/SUM($V19:$AA19), 2),0)</f>
         <v/>
       </c>
-      <c r="H19" s="54">
+      <c r="H19" s="41">
         <f>IF(SUM($V19:$AA19), ROUND(AA19/SUM($V19:$AA19), 2),0)</f>
         <v/>
       </c>
@@ -7389,27 +7393,27 @@
       <c r="B20" s="26" t="n">
         <v>95</v>
       </c>
-      <c r="C20" s="54">
+      <c r="C20" s="41">
         <f>IF(SUM($V20:$AA20), ROUND(V20/SUM($V20:$AA20), 2),0)</f>
         <v/>
       </c>
-      <c r="D20" s="54">
+      <c r="D20" s="41">
         <f>IF(SUM($V20:$AA20), ROUND(W20/SUM($V20:$AA20), 2),0)</f>
         <v/>
       </c>
-      <c r="E20" s="54">
+      <c r="E20" s="41">
         <f>IF(SUM($V20:$AA20), ROUND(X20/SUM($V20:$AA20), 2),0)</f>
         <v/>
       </c>
-      <c r="F20" s="54">
+      <c r="F20" s="41">
         <f>IF(SUM($V20:$AA20), ROUND(Y20/SUM($V20:$AA20), 2),0)</f>
         <v/>
       </c>
-      <c r="G20" s="54">
+      <c r="G20" s="41">
         <f>IF(SUM($V20:$AA20), ROUND(Z20/SUM($V20:$AA20), 2),0)</f>
         <v/>
       </c>
-      <c r="H20" s="54">
+      <c r="H20" s="41">
         <f>IF(SUM($V20:$AA20), ROUND(AA20/SUM($V20:$AA20), 2),0)</f>
         <v/>
       </c>
@@ -7471,27 +7475,27 @@
       <c r="B21" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="C21" s="54">
+      <c r="C21" s="41">
         <f>IF(SUM($V21:$AA21), ROUND(V21/SUM($V21:$AA21), 2),0)</f>
         <v/>
       </c>
-      <c r="D21" s="54">
+      <c r="D21" s="41">
         <f>IF(SUM($V21:$AA21), ROUND(W21/SUM($V21:$AA21), 2),0)</f>
         <v/>
       </c>
-      <c r="E21" s="54">
+      <c r="E21" s="41">
         <f>IF(SUM($V21:$AA21), ROUND(X21/SUM($V21:$AA21), 2),0)</f>
         <v/>
       </c>
-      <c r="F21" s="54">
+      <c r="F21" s="41">
         <f>IF(SUM($V21:$AA21), ROUND(Y21/SUM($V21:$AA21), 2),0)</f>
         <v/>
       </c>
-      <c r="G21" s="54">
+      <c r="G21" s="41">
         <f>IF(SUM($V21:$AA21), ROUND(Z21/SUM($V21:$AA21), 2),0)</f>
         <v/>
       </c>
-      <c r="H21" s="54">
+      <c r="H21" s="41">
         <f>IF(SUM($V21:$AA21), ROUND(AA21/SUM($V21:$AA21), 2),0)</f>
         <v/>
       </c>
@@ -7553,27 +7557,27 @@
       <c r="B22" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="C22" s="54">
+      <c r="C22" s="41">
         <f>IF(SUM($V22:$AA22), ROUND(V22/SUM($V22:$AA22), 2),0)</f>
         <v/>
       </c>
-      <c r="D22" s="54">
+      <c r="D22" s="41">
         <f>IF(SUM($V22:$AA22), ROUND(W22/SUM($V22:$AA22), 2),0)</f>
         <v/>
       </c>
-      <c r="E22" s="54">
+      <c r="E22" s="41">
         <f>IF(SUM($V22:$AA22), ROUND(X22/SUM($V22:$AA22), 2),0)</f>
         <v/>
       </c>
-      <c r="F22" s="54">
+      <c r="F22" s="41">
         <f>IF(SUM($V22:$AA22), ROUND(Y22/SUM($V22:$AA22), 2),0)</f>
         <v/>
       </c>
-      <c r="G22" s="54">
+      <c r="G22" s="41">
         <f>IF(SUM($V22:$AA22), ROUND(Z22/SUM($V22:$AA22), 2),0)</f>
         <v/>
       </c>
-      <c r="H22" s="54">
+      <c r="H22" s="41">
         <f>IF(SUM($V22:$AA22), ROUND(AA22/SUM($V22:$AA22), 2),0)</f>
         <v/>
       </c>
@@ -7635,27 +7639,27 @@
       <c r="B23" s="26" t="n">
         <v>38</v>
       </c>
-      <c r="C23" s="54">
+      <c r="C23" s="41">
         <f>IF(SUM($V23:$AA23), ROUND(V23/SUM($V23:$AA23), 2),0)</f>
         <v/>
       </c>
-      <c r="D23" s="54">
+      <c r="D23" s="41">
         <f>IF(SUM($V23:$AA23), ROUND(W23/SUM($V23:$AA23), 2),0)</f>
         <v/>
       </c>
-      <c r="E23" s="54">
+      <c r="E23" s="41">
         <f>IF(SUM($V23:$AA23), ROUND(X23/SUM($V23:$AA23), 2),0)</f>
         <v/>
       </c>
-      <c r="F23" s="54">
+      <c r="F23" s="41">
         <f>IF(SUM($V23:$AA23), ROUND(Y23/SUM($V23:$AA23), 2),0)</f>
         <v/>
       </c>
-      <c r="G23" s="54">
+      <c r="G23" s="41">
         <f>IF(SUM($V23:$AA23), ROUND(Z23/SUM($V23:$AA23), 2),0)</f>
         <v/>
       </c>
-      <c r="H23" s="54">
+      <c r="H23" s="41">
         <f>IF(SUM($V23:$AA23), ROUND(AA23/SUM($V23:$AA23), 2),0)</f>
         <v/>
       </c>
@@ -7717,27 +7721,27 @@
       <c r="B24" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C24" s="54">
+      <c r="C24" s="41">
         <f>IF(SUM($V24:$AA24), ROUND(V24/SUM($V24:$AA24), 2),0)</f>
         <v/>
       </c>
-      <c r="D24" s="54">
+      <c r="D24" s="41">
         <f>IF(SUM($V24:$AA24), ROUND(W24/SUM($V24:$AA24), 2),0)</f>
         <v/>
       </c>
-      <c r="E24" s="54">
+      <c r="E24" s="41">
         <f>IF(SUM($V24:$AA24), ROUND(X24/SUM($V24:$AA24), 2),0)</f>
         <v/>
       </c>
-      <c r="F24" s="54">
+      <c r="F24" s="41">
         <f>IF(SUM($V24:$AA24), ROUND(Y24/SUM($V24:$AA24), 2),0)</f>
         <v/>
       </c>
-      <c r="G24" s="54">
+      <c r="G24" s="41">
         <f>IF(SUM($V24:$AA24), ROUND(Z24/SUM($V24:$AA24), 2),0)</f>
         <v/>
       </c>
-      <c r="H24" s="54">
+      <c r="H24" s="41">
         <f>IF(SUM($V24:$AA24), ROUND(AA24/SUM($V24:$AA24), 2),0)</f>
         <v/>
       </c>
@@ -7799,27 +7803,27 @@
       <c r="B25" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C25" s="54">
+      <c r="C25" s="41">
         <f>IF(SUM($V25:$AA25), ROUND(V25/SUM($V25:$AA25), 2),0)</f>
         <v/>
       </c>
-      <c r="D25" s="54">
+      <c r="D25" s="41">
         <f>IF(SUM($V25:$AA25), ROUND(W25/SUM($V25:$AA25), 2),0)</f>
         <v/>
       </c>
-      <c r="E25" s="54">
+      <c r="E25" s="41">
         <f>IF(SUM($V25:$AA25), ROUND(X25/SUM($V25:$AA25), 2),0)</f>
         <v/>
       </c>
-      <c r="F25" s="54">
+      <c r="F25" s="41">
         <f>IF(SUM($V25:$AA25), ROUND(Y25/SUM($V25:$AA25), 2),0)</f>
         <v/>
       </c>
-      <c r="G25" s="54">
+      <c r="G25" s="41">
         <f>IF(SUM($V25:$AA25), ROUND(Z25/SUM($V25:$AA25), 2),0)</f>
         <v/>
       </c>
-      <c r="H25" s="54">
+      <c r="H25" s="41">
         <f>IF(SUM($V25:$AA25), ROUND(AA25/SUM($V25:$AA25), 2),0)</f>
         <v/>
       </c>
@@ -7881,27 +7885,27 @@
       <c r="B26" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C26" s="54">
+      <c r="C26" s="41">
         <f>IF(SUM($V26:$AA26), ROUND(V26/SUM($V26:$AA26), 2),0)</f>
         <v/>
       </c>
-      <c r="D26" s="54">
+      <c r="D26" s="41">
         <f>IF(SUM($V26:$AA26), ROUND(W26/SUM($V26:$AA26), 2),0)</f>
         <v/>
       </c>
-      <c r="E26" s="54">
+      <c r="E26" s="41">
         <f>IF(SUM($V26:$AA26), ROUND(X26/SUM($V26:$AA26), 2),0)</f>
         <v/>
       </c>
-      <c r="F26" s="54">
+      <c r="F26" s="41">
         <f>IF(SUM($V26:$AA26), ROUND(Y26/SUM($V26:$AA26), 2),0)</f>
         <v/>
       </c>
-      <c r="G26" s="54">
+      <c r="G26" s="41">
         <f>IF(SUM($V26:$AA26), ROUND(Z26/SUM($V26:$AA26), 2),0)</f>
         <v/>
       </c>
-      <c r="H26" s="54">
+      <c r="H26" s="41">
         <f>IF(SUM($V26:$AA26), ROUND(AA26/SUM($V26:$AA26), 2),0)</f>
         <v/>
       </c>
@@ -7963,27 +7967,27 @@
       <c r="B27" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C27" s="54">
+      <c r="C27" s="41">
         <f>IF(SUM($V27:$AA27), ROUND(V27/SUM($V27:$AA27), 2),0)</f>
         <v/>
       </c>
-      <c r="D27" s="54">
+      <c r="D27" s="41">
         <f>IF(SUM($V27:$AA27), ROUND(W27/SUM($V27:$AA27), 2),0)</f>
         <v/>
       </c>
-      <c r="E27" s="54">
+      <c r="E27" s="41">
         <f>IF(SUM($V27:$AA27), ROUND(X27/SUM($V27:$AA27), 2),0)</f>
         <v/>
       </c>
-      <c r="F27" s="54">
+      <c r="F27" s="41">
         <f>IF(SUM($V27:$AA27), ROUND(Y27/SUM($V27:$AA27), 2),0)</f>
         <v/>
       </c>
-      <c r="G27" s="54">
+      <c r="G27" s="41">
         <f>IF(SUM($V27:$AA27), ROUND(Z27/SUM($V27:$AA27), 2),0)</f>
         <v/>
       </c>
-      <c r="H27" s="54">
+      <c r="H27" s="41">
         <f>IF(SUM($V27:$AA27), ROUND(AA27/SUM($V27:$AA27), 2),0)</f>
         <v/>
       </c>
@@ -8045,27 +8049,27 @@
       <c r="B28" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C28" s="54">
+      <c r="C28" s="41">
         <f>IF(SUM($V28:$AA28), ROUND(V28/SUM($V28:$AA28), 2),0)</f>
         <v/>
       </c>
-      <c r="D28" s="54">
+      <c r="D28" s="41">
         <f>IF(SUM($V28:$AA28), ROUND(W28/SUM($V28:$AA28), 2),0)</f>
         <v/>
       </c>
-      <c r="E28" s="54">
+      <c r="E28" s="41">
         <f>IF(SUM($V28:$AA28), ROUND(X28/SUM($V28:$AA28), 2),0)</f>
         <v/>
       </c>
-      <c r="F28" s="54">
+      <c r="F28" s="41">
         <f>IF(SUM($V28:$AA28), ROUND(Y28/SUM($V28:$AA28), 2),0)</f>
         <v/>
       </c>
-      <c r="G28" s="54">
+      <c r="G28" s="41">
         <f>IF(SUM($V28:$AA28), ROUND(Z28/SUM($V28:$AA28), 2),0)</f>
         <v/>
       </c>
-      <c r="H28" s="54">
+      <c r="H28" s="41">
         <f>IF(SUM($V28:$AA28), ROUND(AA28/SUM($V28:$AA28), 2),0)</f>
         <v/>
       </c>
@@ -8127,27 +8131,27 @@
       <c r="B29" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C29" s="54">
+      <c r="C29" s="41">
         <f>IF(SUM($V29:$AA29), ROUND(V29/SUM($V29:$AA29), 2),0)</f>
         <v/>
       </c>
-      <c r="D29" s="54">
+      <c r="D29" s="41">
         <f>IF(SUM($V29:$AA29), ROUND(W29/SUM($V29:$AA29), 2),0)</f>
         <v/>
       </c>
-      <c r="E29" s="54">
+      <c r="E29" s="41">
         <f>IF(SUM($V29:$AA29), ROUND(X29/SUM($V29:$AA29), 2),0)</f>
         <v/>
       </c>
-      <c r="F29" s="54">
+      <c r="F29" s="41">
         <f>IF(SUM($V29:$AA29), ROUND(Y29/SUM($V29:$AA29), 2),0)</f>
         <v/>
       </c>
-      <c r="G29" s="54">
+      <c r="G29" s="41">
         <f>IF(SUM($V29:$AA29), ROUND(Z29/SUM($V29:$AA29), 2),0)</f>
         <v/>
       </c>
-      <c r="H29" s="54">
+      <c r="H29" s="41">
         <f>IF(SUM($V29:$AA29), ROUND(AA29/SUM($V29:$AA29), 2),0)</f>
         <v/>
       </c>
@@ -8209,27 +8213,27 @@
       <c r="B30" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C30" s="54">
+      <c r="C30" s="41">
         <f>IF(SUM($V30:$AA30), ROUND(V30/SUM($V30:$AA30), 2),0)</f>
         <v/>
       </c>
-      <c r="D30" s="54">
+      <c r="D30" s="41">
         <f>IF(SUM($V30:$AA30), ROUND(W30/SUM($V30:$AA30), 2),0)</f>
         <v/>
       </c>
-      <c r="E30" s="54">
+      <c r="E30" s="41">
         <f>IF(SUM($V30:$AA30), ROUND(X30/SUM($V30:$AA30), 2),0)</f>
         <v/>
       </c>
-      <c r="F30" s="54">
+      <c r="F30" s="41">
         <f>IF(SUM($V30:$AA30), ROUND(Y30/SUM($V30:$AA30), 2),0)</f>
         <v/>
       </c>
-      <c r="G30" s="54">
+      <c r="G30" s="41">
         <f>IF(SUM($V30:$AA30), ROUND(Z30/SUM($V30:$AA30), 2),0)</f>
         <v/>
       </c>
-      <c r="H30" s="54">
+      <c r="H30" s="41">
         <f>IF(SUM($V30:$AA30), ROUND(AA30/SUM($V30:$AA30), 2),0)</f>
         <v/>
       </c>
@@ -8291,27 +8295,27 @@
       <c r="B31" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C31" s="54">
+      <c r="C31" s="41">
         <f>IF(SUM($V31:$AA31), ROUND(V31/SUM($V31:$AA31), 2),0)</f>
         <v/>
       </c>
-      <c r="D31" s="54">
+      <c r="D31" s="41">
         <f>IF(SUM($V31:$AA31), ROUND(W31/SUM($V31:$AA31), 2),0)</f>
         <v/>
       </c>
-      <c r="E31" s="54">
+      <c r="E31" s="41">
         <f>IF(SUM($V31:$AA31), ROUND(X31/SUM($V31:$AA31), 2),0)</f>
         <v/>
       </c>
-      <c r="F31" s="54">
+      <c r="F31" s="41">
         <f>IF(SUM($V31:$AA31), ROUND(Y31/SUM($V31:$AA31), 2),0)</f>
         <v/>
       </c>
-      <c r="G31" s="54">
+      <c r="G31" s="41">
         <f>IF(SUM($V31:$AA31), ROUND(Z31/SUM($V31:$AA31), 2),0)</f>
         <v/>
       </c>
-      <c r="H31" s="54">
+      <c r="H31" s="41">
         <f>IF(SUM($V31:$AA31), ROUND(AA31/SUM($V31:$AA31), 2),0)</f>
         <v/>
       </c>
@@ -8373,27 +8377,27 @@
       <c r="B32" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C32" s="54">
+      <c r="C32" s="41">
         <f>IF(SUM($V32:$AA32), ROUND(V32/SUM($V32:$AA32), 2),0)</f>
         <v/>
       </c>
-      <c r="D32" s="54">
+      <c r="D32" s="41">
         <f>IF(SUM($V32:$AA32), ROUND(W32/SUM($V32:$AA32), 2),0)</f>
         <v/>
       </c>
-      <c r="E32" s="54">
+      <c r="E32" s="41">
         <f>IF(SUM($V32:$AA32), ROUND(X32/SUM($V32:$AA32), 2),0)</f>
         <v/>
       </c>
-      <c r="F32" s="54">
+      <c r="F32" s="41">
         <f>IF(SUM($V32:$AA32), ROUND(Y32/SUM($V32:$AA32), 2),0)</f>
         <v/>
       </c>
-      <c r="G32" s="54">
+      <c r="G32" s="41">
         <f>IF(SUM($V32:$AA32), ROUND(Z32/SUM($V32:$AA32), 2),0)</f>
         <v/>
       </c>
-      <c r="H32" s="54">
+      <c r="H32" s="41">
         <f>IF(SUM($V32:$AA32), ROUND(AA32/SUM($V32:$AA32), 2),0)</f>
         <v/>
       </c>
@@ -8455,27 +8459,27 @@
       <c r="B33" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C33" s="54">
+      <c r="C33" s="41">
         <f>IF(SUM($V33:$AA33), ROUND(V33/SUM($V33:$AA33), 2),0)</f>
         <v/>
       </c>
-      <c r="D33" s="54">
+      <c r="D33" s="41">
         <f>IF(SUM($V33:$AA33), ROUND(W33/SUM($V33:$AA33), 2),0)</f>
         <v/>
       </c>
-      <c r="E33" s="54">
+      <c r="E33" s="41">
         <f>IF(SUM($V33:$AA33), ROUND(X33/SUM($V33:$AA33), 2),0)</f>
         <v/>
       </c>
-      <c r="F33" s="54">
+      <c r="F33" s="41">
         <f>IF(SUM($V33:$AA33), ROUND(Y33/SUM($V33:$AA33), 2),0)</f>
         <v/>
       </c>
-      <c r="G33" s="54">
+      <c r="G33" s="41">
         <f>IF(SUM($V33:$AA33), ROUND(Z33/SUM($V33:$AA33), 2),0)</f>
         <v/>
       </c>
-      <c r="H33" s="54">
+      <c r="H33" s="41">
         <f>IF(SUM($V33:$AA33), ROUND(AA33/SUM($V33:$AA33), 2),0)</f>
         <v/>
       </c>
@@ -8537,27 +8541,27 @@
       <c r="B34" s="26" t="n">
         <v>620</v>
       </c>
-      <c r="C34" s="54">
+      <c r="C34" s="41">
         <f>IF(SUM($V34:$AA34), ROUND(V34/SUM($V34:$AA34), 2),0)</f>
         <v/>
       </c>
-      <c r="D34" s="54">
+      <c r="D34" s="41">
         <f>IF(SUM($V34:$AA34), ROUND(W34/SUM($V34:$AA34), 2),0)</f>
         <v/>
       </c>
-      <c r="E34" s="54">
+      <c r="E34" s="41">
         <f>IF(SUM($V34:$AA34), ROUND(X34/SUM($V34:$AA34), 2),0)</f>
         <v/>
       </c>
-      <c r="F34" s="54">
+      <c r="F34" s="41">
         <f>IF(SUM($V34:$AA34), ROUND(Y34/SUM($V34:$AA34), 2),0)</f>
         <v/>
       </c>
-      <c r="G34" s="54">
+      <c r="G34" s="41">
         <f>IF(SUM($V34:$AA34), ROUND(Z34/SUM($V34:$AA34), 2),0)</f>
         <v/>
       </c>
-      <c r="H34" s="54">
+      <c r="H34" s="41">
         <f>IF(SUM($V34:$AA34), ROUND(AA34/SUM($V34:$AA34), 2),0)</f>
         <v/>
       </c>
@@ -8621,27 +8625,27 @@
       <c r="B35" s="26" t="n">
         <v>39</v>
       </c>
-      <c r="C35" s="54">
+      <c r="C35" s="41">
         <f>IF(SUM($V35:$AA35), ROUND(V35/SUM($V35:$AA35), 2),0)</f>
         <v/>
       </c>
-      <c r="D35" s="54">
+      <c r="D35" s="41">
         <f>IF(SUM($V35:$AA35), ROUND(W35/SUM($V35:$AA35), 2),0)</f>
         <v/>
       </c>
-      <c r="E35" s="54">
+      <c r="E35" s="41">
         <f>IF(SUM($V35:$AA35), ROUND(X35/SUM($V35:$AA35), 2),0)</f>
         <v/>
       </c>
-      <c r="F35" s="54">
+      <c r="F35" s="41">
         <f>IF(SUM($V35:$AA35), ROUND(Y35/SUM($V35:$AA35), 2),0)</f>
         <v/>
       </c>
-      <c r="G35" s="54">
+      <c r="G35" s="41">
         <f>IF(SUM($V35:$AA35), ROUND(Z35/SUM($V35:$AA35), 2),0)</f>
         <v/>
       </c>
-      <c r="H35" s="54">
+      <c r="H35" s="41">
         <f>IF(SUM($V35:$AA35), ROUND(AA35/SUM($V35:$AA35), 2),0)</f>
         <v/>
       </c>
@@ -8703,27 +8707,27 @@
       <c r="B36" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C36" s="54">
+      <c r="C36" s="41">
         <f>IF(SUM($V36:$AA36), ROUND(V36/SUM($V36:$AA36), 2),0)</f>
         <v/>
       </c>
-      <c r="D36" s="54">
+      <c r="D36" s="41">
         <f>IF(SUM($V36:$AA36), ROUND(W36/SUM($V36:$AA36), 2),0)</f>
         <v/>
       </c>
-      <c r="E36" s="54">
+      <c r="E36" s="41">
         <f>IF(SUM($V36:$AA36), ROUND(X36/SUM($V36:$AA36), 2),0)</f>
         <v/>
       </c>
-      <c r="F36" s="54">
+      <c r="F36" s="41">
         <f>IF(SUM($V36:$AA36), ROUND(Y36/SUM($V36:$AA36), 2),0)</f>
         <v/>
       </c>
-      <c r="G36" s="54">
+      <c r="G36" s="41">
         <f>IF(SUM($V36:$AA36), ROUND(Z36/SUM($V36:$AA36), 2),0)</f>
         <v/>
       </c>
-      <c r="H36" s="54">
+      <c r="H36" s="41">
         <f>IF(SUM($V36:$AA36), ROUND(AA36/SUM($V36:$AA36), 2),0)</f>
         <v/>
       </c>
@@ -8785,27 +8789,27 @@
       <c r="B37" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="C37" s="54">
+      <c r="C37" s="41">
         <f>IF(SUM($V37:$AA37), ROUND(V37/SUM($V37:$AA37), 2),0)</f>
         <v/>
       </c>
-      <c r="D37" s="54">
+      <c r="D37" s="41">
         <f>IF(SUM($V37:$AA37), ROUND(W37/SUM($V37:$AA37), 2),0)</f>
         <v/>
       </c>
-      <c r="E37" s="54">
+      <c r="E37" s="41">
         <f>IF(SUM($V37:$AA37), ROUND(X37/SUM($V37:$AA37), 2),0)</f>
         <v/>
       </c>
-      <c r="F37" s="54">
+      <c r="F37" s="41">
         <f>IF(SUM($V37:$AA37), ROUND(Y37/SUM($V37:$AA37), 2),0)</f>
         <v/>
       </c>
-      <c r="G37" s="54">
+      <c r="G37" s="41">
         <f>IF(SUM($V37:$AA37), ROUND(Z37/SUM($V37:$AA37), 2),0)</f>
         <v/>
       </c>
-      <c r="H37" s="54">
+      <c r="H37" s="41">
         <f>IF(SUM($V37:$AA37), ROUND(AA37/SUM($V37:$AA37), 2),0)</f>
         <v/>
       </c>
@@ -8867,27 +8871,27 @@
       <c r="B38" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C38" s="54">
+      <c r="C38" s="41">
         <f>IF(SUM($V38:$AA38), ROUND(V38/SUM($V38:$AA38), 2),0)</f>
         <v/>
       </c>
-      <c r="D38" s="54">
+      <c r="D38" s="41">
         <f>IF(SUM($V38:$AA38), ROUND(W38/SUM($V38:$AA38), 2),0)</f>
         <v/>
       </c>
-      <c r="E38" s="54">
+      <c r="E38" s="41">
         <f>IF(SUM($V38:$AA38), ROUND(X38/SUM($V38:$AA38), 2),0)</f>
         <v/>
       </c>
-      <c r="F38" s="54">
+      <c r="F38" s="41">
         <f>IF(SUM($V38:$AA38), ROUND(Y38/SUM($V38:$AA38), 2),0)</f>
         <v/>
       </c>
-      <c r="G38" s="54">
+      <c r="G38" s="41">
         <f>IF(SUM($V38:$AA38), ROUND(Z38/SUM($V38:$AA38), 2),0)</f>
         <v/>
       </c>
-      <c r="H38" s="54">
+      <c r="H38" s="41">
         <f>IF(SUM($V38:$AA38), ROUND(AA38/SUM($V38:$AA38), 2),0)</f>
         <v/>
       </c>
@@ -8949,27 +8953,27 @@
       <c r="B39" s="26" t="n">
         <v>23</v>
       </c>
-      <c r="C39" s="54">
+      <c r="C39" s="41">
         <f>IF(SUM($V39:$AA39), ROUND(V39/SUM($V39:$AA39), 2),0)</f>
         <v/>
       </c>
-      <c r="D39" s="54">
+      <c r="D39" s="41">
         <f>IF(SUM($V39:$AA39), ROUND(W39/SUM($V39:$AA39), 2),0)</f>
         <v/>
       </c>
-      <c r="E39" s="54">
+      <c r="E39" s="41">
         <f>IF(SUM($V39:$AA39), ROUND(X39/SUM($V39:$AA39), 2),0)</f>
         <v/>
       </c>
-      <c r="F39" s="54">
+      <c r="F39" s="41">
         <f>IF(SUM($V39:$AA39), ROUND(Y39/SUM($V39:$AA39), 2),0)</f>
         <v/>
       </c>
-      <c r="G39" s="54">
+      <c r="G39" s="41">
         <f>IF(SUM($V39:$AA39), ROUND(Z39/SUM($V39:$AA39), 2),0)</f>
         <v/>
       </c>
-      <c r="H39" s="54">
+      <c r="H39" s="41">
         <f>IF(SUM($V39:$AA39), ROUND(AA39/SUM($V39:$AA39), 2),0)</f>
         <v/>
       </c>
@@ -9031,27 +9035,27 @@
       <c r="B40" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C40" s="54">
+      <c r="C40" s="41">
         <f>IF(SUM($V40:$AA40), ROUND(V40/SUM($V40:$AA40), 2),0)</f>
         <v/>
       </c>
-      <c r="D40" s="54">
+      <c r="D40" s="41">
         <f>IF(SUM($V40:$AA40), ROUND(W40/SUM($V40:$AA40), 2),0)</f>
         <v/>
       </c>
-      <c r="E40" s="54">
+      <c r="E40" s="41">
         <f>IF(SUM($V40:$AA40), ROUND(X40/SUM($V40:$AA40), 2),0)</f>
         <v/>
       </c>
-      <c r="F40" s="54">
+      <c r="F40" s="41">
         <f>IF(SUM($V40:$AA40), ROUND(Y40/SUM($V40:$AA40), 2),0)</f>
         <v/>
       </c>
-      <c r="G40" s="54">
+      <c r="G40" s="41">
         <f>IF(SUM($V40:$AA40), ROUND(Z40/SUM($V40:$AA40), 2),0)</f>
         <v/>
       </c>
-      <c r="H40" s="54">
+      <c r="H40" s="41">
         <f>IF(SUM($V40:$AA40), ROUND(AA40/SUM($V40:$AA40), 2),0)</f>
         <v/>
       </c>
@@ -9113,27 +9117,27 @@
       <c r="B41" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C41" s="54">
+      <c r="C41" s="41">
         <f>IF(SUM($V41:$AA41), ROUND(V41/SUM($V41:$AA41), 2),0)</f>
         <v/>
       </c>
-      <c r="D41" s="54">
+      <c r="D41" s="41">
         <f>IF(SUM($V41:$AA41), ROUND(W41/SUM($V41:$AA41), 2),0)</f>
         <v/>
       </c>
-      <c r="E41" s="54">
+      <c r="E41" s="41">
         <f>IF(SUM($V41:$AA41), ROUND(X41/SUM($V41:$AA41), 2),0)</f>
         <v/>
       </c>
-      <c r="F41" s="54">
+      <c r="F41" s="41">
         <f>IF(SUM($V41:$AA41), ROUND(Y41/SUM($V41:$AA41), 2),0)</f>
         <v/>
       </c>
-      <c r="G41" s="54">
+      <c r="G41" s="41">
         <f>IF(SUM($V41:$AA41), ROUND(Z41/SUM($V41:$AA41), 2),0)</f>
         <v/>
       </c>
-      <c r="H41" s="54">
+      <c r="H41" s="41">
         <f>IF(SUM($V41:$AA41), ROUND(AA41/SUM($V41:$AA41), 2),0)</f>
         <v/>
       </c>
@@ -9195,27 +9199,27 @@
       <c r="B42" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C42" s="54">
+      <c r="C42" s="41">
         <f>IF(SUM($V42:$AA42), ROUND(V42/SUM($V42:$AA42), 2),0)</f>
         <v/>
       </c>
-      <c r="D42" s="54">
+      <c r="D42" s="41">
         <f>IF(SUM($V42:$AA42), ROUND(W42/SUM($V42:$AA42), 2),0)</f>
         <v/>
       </c>
-      <c r="E42" s="54">
+      <c r="E42" s="41">
         <f>IF(SUM($V42:$AA42), ROUND(X42/SUM($V42:$AA42), 2),0)</f>
         <v/>
       </c>
-      <c r="F42" s="54">
+      <c r="F42" s="41">
         <f>IF(SUM($V42:$AA42), ROUND(Y42/SUM($V42:$AA42), 2),0)</f>
         <v/>
       </c>
-      <c r="G42" s="54">
+      <c r="G42" s="41">
         <f>IF(SUM($V42:$AA42), ROUND(Z42/SUM($V42:$AA42), 2),0)</f>
         <v/>
       </c>
-      <c r="H42" s="54">
+      <c r="H42" s="41">
         <f>IF(SUM($V42:$AA42), ROUND(AA42/SUM($V42:$AA42), 2),0)</f>
         <v/>
       </c>
@@ -9277,27 +9281,27 @@
       <c r="B43" s="26" t="n">
         <v>28</v>
       </c>
-      <c r="C43" s="54">
+      <c r="C43" s="41">
         <f>IF(SUM($V43:$AA43), ROUND(V43/SUM($V43:$AA43), 2),0)</f>
         <v/>
       </c>
-      <c r="D43" s="54">
+      <c r="D43" s="41">
         <f>IF(SUM($V43:$AA43), ROUND(W43/SUM($V43:$AA43), 2),0)</f>
         <v/>
       </c>
-      <c r="E43" s="54">
+      <c r="E43" s="41">
         <f>IF(SUM($V43:$AA43), ROUND(X43/SUM($V43:$AA43), 2),0)</f>
         <v/>
       </c>
-      <c r="F43" s="54">
+      <c r="F43" s="41">
         <f>IF(SUM($V43:$AA43), ROUND(Y43/SUM($V43:$AA43), 2),0)</f>
         <v/>
       </c>
-      <c r="G43" s="54">
+      <c r="G43" s="41">
         <f>IF(SUM($V43:$AA43), ROUND(Z43/SUM($V43:$AA43), 2),0)</f>
         <v/>
       </c>
-      <c r="H43" s="54">
+      <c r="H43" s="41">
         <f>IF(SUM($V43:$AA43), ROUND(AA43/SUM($V43:$AA43), 2),0)</f>
         <v/>
       </c>
@@ -9359,27 +9363,27 @@
       <c r="B44" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C44" s="54">
+      <c r="C44" s="41">
         <f>IF(SUM($V44:$AA44), ROUND(V44/SUM($V44:$AA44), 2),0)</f>
         <v/>
       </c>
-      <c r="D44" s="54">
+      <c r="D44" s="41">
         <f>IF(SUM($V44:$AA44), ROUND(W44/SUM($V44:$AA44), 2),0)</f>
         <v/>
       </c>
-      <c r="E44" s="54">
+      <c r="E44" s="41">
         <f>IF(SUM($V44:$AA44), ROUND(X44/SUM($V44:$AA44), 2),0)</f>
         <v/>
       </c>
-      <c r="F44" s="54">
+      <c r="F44" s="41">
         <f>IF(SUM($V44:$AA44), ROUND(Y44/SUM($V44:$AA44), 2),0)</f>
         <v/>
       </c>
-      <c r="G44" s="54">
+      <c r="G44" s="41">
         <f>IF(SUM($V44:$AA44), ROUND(Z44/SUM($V44:$AA44), 2),0)</f>
         <v/>
       </c>
-      <c r="H44" s="54">
+      <c r="H44" s="41">
         <f>IF(SUM($V44:$AA44), ROUND(AA44/SUM($V44:$AA44), 2),0)</f>
         <v/>
       </c>
@@ -9441,27 +9445,27 @@
       <c r="B45" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C45" s="54">
+      <c r="C45" s="41">
         <f>IF(SUM($V45:$AA45), ROUND(V45/SUM($V45:$AA45), 2),0)</f>
         <v/>
       </c>
-      <c r="D45" s="54">
+      <c r="D45" s="41">
         <f>IF(SUM($V45:$AA45), ROUND(W45/SUM($V45:$AA45), 2),0)</f>
         <v/>
       </c>
-      <c r="E45" s="54">
+      <c r="E45" s="41">
         <f>IF(SUM($V45:$AA45), ROUND(X45/SUM($V45:$AA45), 2),0)</f>
         <v/>
       </c>
-      <c r="F45" s="54">
+      <c r="F45" s="41">
         <f>IF(SUM($V45:$AA45), ROUND(Y45/SUM($V45:$AA45), 2),0)</f>
         <v/>
       </c>
-      <c r="G45" s="54">
+      <c r="G45" s="41">
         <f>IF(SUM($V45:$AA45), ROUND(Z45/SUM($V45:$AA45), 2),0)</f>
         <v/>
       </c>
-      <c r="H45" s="54">
+      <c r="H45" s="41">
         <f>IF(SUM($V45:$AA45), ROUND(AA45/SUM($V45:$AA45), 2),0)</f>
         <v/>
       </c>
@@ -9523,27 +9527,27 @@
       <c r="B46" s="26" t="n">
         <v>56</v>
       </c>
-      <c r="C46" s="54">
+      <c r="C46" s="41">
         <f>IF(SUM($V46:$AA46), ROUND(V46/SUM($V46:$AA46), 2),0)</f>
         <v/>
       </c>
-      <c r="D46" s="54">
+      <c r="D46" s="41">
         <f>IF(SUM($V46:$AA46), ROUND(W46/SUM($V46:$AA46), 2),0)</f>
         <v/>
       </c>
-      <c r="E46" s="54">
+      <c r="E46" s="41">
         <f>IF(SUM($V46:$AA46), ROUND(X46/SUM($V46:$AA46), 2),0)</f>
         <v/>
       </c>
-      <c r="F46" s="54">
+      <c r="F46" s="41">
         <f>IF(SUM($V46:$AA46), ROUND(Y46/SUM($V46:$AA46), 2),0)</f>
         <v/>
       </c>
-      <c r="G46" s="54">
+      <c r="G46" s="41">
         <f>IF(SUM($V46:$AA46), ROUND(Z46/SUM($V46:$AA46), 2),0)</f>
         <v/>
       </c>
-      <c r="H46" s="54">
+      <c r="H46" s="41">
         <f>IF(SUM($V46:$AA46), ROUND(AA46/SUM($V46:$AA46), 2),0)</f>
         <v/>
       </c>
@@ -9605,27 +9609,27 @@
       <c r="B47" s="26" t="n">
         <v>904</v>
       </c>
-      <c r="C47" s="54">
+      <c r="C47" s="41">
         <f>IF(SUM($V47:$AA47), ROUND(V47/SUM($V47:$AA47), 2),0)</f>
         <v/>
       </c>
-      <c r="D47" s="54">
+      <c r="D47" s="41">
         <f>IF(SUM($V47:$AA47), ROUND(W47/SUM($V47:$AA47), 2),0)</f>
         <v/>
       </c>
-      <c r="E47" s="54">
+      <c r="E47" s="41">
         <f>IF(SUM($V47:$AA47), ROUND(X47/SUM($V47:$AA47), 2),0)</f>
         <v/>
       </c>
-      <c r="F47" s="54">
+      <c r="F47" s="41">
         <f>IF(SUM($V47:$AA47), ROUND(Y47/SUM($V47:$AA47), 2),0)</f>
         <v/>
       </c>
-      <c r="G47" s="54">
+      <c r="G47" s="41">
         <f>IF(SUM($V47:$AA47), ROUND(Z47/SUM($V47:$AA47), 2),0)</f>
         <v/>
       </c>
-      <c r="H47" s="54">
+      <c r="H47" s="41">
         <f>IF(SUM($V47:$AA47), ROUND(AA47/SUM($V47:$AA47), 2),0)</f>
         <v/>
       </c>
@@ -9689,27 +9693,27 @@
       <c r="B48" s="26" t="n">
         <v>92</v>
       </c>
-      <c r="C48" s="54">
+      <c r="C48" s="41">
         <f>IF(SUM($V48:$AA48), ROUND(V48/SUM($V48:$AA48), 2),0)</f>
         <v/>
       </c>
-      <c r="D48" s="54">
+      <c r="D48" s="41">
         <f>IF(SUM($V48:$AA48), ROUND(W48/SUM($V48:$AA48), 2),0)</f>
         <v/>
       </c>
-      <c r="E48" s="54">
+      <c r="E48" s="41">
         <f>IF(SUM($V48:$AA48), ROUND(X48/SUM($V48:$AA48), 2),0)</f>
         <v/>
       </c>
-      <c r="F48" s="54">
+      <c r="F48" s="41">
         <f>IF(SUM($V48:$AA48), ROUND(Y48/SUM($V48:$AA48), 2),0)</f>
         <v/>
       </c>
-      <c r="G48" s="54">
+      <c r="G48" s="41">
         <f>IF(SUM($V48:$AA48), ROUND(Z48/SUM($V48:$AA48), 2),0)</f>
         <v/>
       </c>
-      <c r="H48" s="54">
+      <c r="H48" s="41">
         <f>IF(SUM($V48:$AA48), ROUND(AA48/SUM($V48:$AA48), 2),0)</f>
         <v/>
       </c>
@@ -9771,27 +9775,27 @@
       <c r="B49" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="C49" s="54">
+      <c r="C49" s="41">
         <f>IF(SUM($V49:$AA49), ROUND(V49/SUM($V49:$AA49), 2),0)</f>
         <v/>
       </c>
-      <c r="D49" s="54">
+      <c r="D49" s="41">
         <f>IF(SUM($V49:$AA49), ROUND(W49/SUM($V49:$AA49), 2),0)</f>
         <v/>
       </c>
-      <c r="E49" s="54">
+      <c r="E49" s="41">
         <f>IF(SUM($V49:$AA49), ROUND(X49/SUM($V49:$AA49), 2),0)</f>
         <v/>
       </c>
-      <c r="F49" s="54">
+      <c r="F49" s="41">
         <f>IF(SUM($V49:$AA49), ROUND(Y49/SUM($V49:$AA49), 2),0)</f>
         <v/>
       </c>
-      <c r="G49" s="54">
+      <c r="G49" s="41">
         <f>IF(SUM($V49:$AA49), ROUND(Z49/SUM($V49:$AA49), 2),0)</f>
         <v/>
       </c>
-      <c r="H49" s="54">
+      <c r="H49" s="41">
         <f>IF(SUM($V49:$AA49), ROUND(AA49/SUM($V49:$AA49), 2),0)</f>
         <v/>
       </c>
@@ -9853,27 +9857,27 @@
       <c r="B50" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C50" s="54">
+      <c r="C50" s="41">
         <f>IF(SUM($V50:$AA50), ROUND(V50/SUM($V50:$AA50), 2),0)</f>
         <v/>
       </c>
-      <c r="D50" s="54">
+      <c r="D50" s="41">
         <f>IF(SUM($V50:$AA50), ROUND(W50/SUM($V50:$AA50), 2),0)</f>
         <v/>
       </c>
-      <c r="E50" s="54">
+      <c r="E50" s="41">
         <f>IF(SUM($V50:$AA50), ROUND(X50/SUM($V50:$AA50), 2),0)</f>
         <v/>
       </c>
-      <c r="F50" s="54">
+      <c r="F50" s="41">
         <f>IF(SUM($V50:$AA50), ROUND(Y50/SUM($V50:$AA50), 2),0)</f>
         <v/>
       </c>
-      <c r="G50" s="54">
+      <c r="G50" s="41">
         <f>IF(SUM($V50:$AA50), ROUND(Z50/SUM($V50:$AA50), 2),0)</f>
         <v/>
       </c>
-      <c r="H50" s="54">
+      <c r="H50" s="41">
         <f>IF(SUM($V50:$AA50), ROUND(AA50/SUM($V50:$AA50), 2),0)</f>
         <v/>
       </c>
@@ -9935,27 +9939,27 @@
       <c r="B51" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C51" s="54">
+      <c r="C51" s="41">
         <f>IF(SUM($V51:$AA51), ROUND(V51/SUM($V51:$AA51), 2),0)</f>
         <v/>
       </c>
-      <c r="D51" s="54">
+      <c r="D51" s="41">
         <f>IF(SUM($V51:$AA51), ROUND(W51/SUM($V51:$AA51), 2),0)</f>
         <v/>
       </c>
-      <c r="E51" s="54">
+      <c r="E51" s="41">
         <f>IF(SUM($V51:$AA51), ROUND(X51/SUM($V51:$AA51), 2),0)</f>
         <v/>
       </c>
-      <c r="F51" s="54">
+      <c r="F51" s="41">
         <f>IF(SUM($V51:$AA51), ROUND(Y51/SUM($V51:$AA51), 2),0)</f>
         <v/>
       </c>
-      <c r="G51" s="54">
+      <c r="G51" s="41">
         <f>IF(SUM($V51:$AA51), ROUND(Z51/SUM($V51:$AA51), 2),0)</f>
         <v/>
       </c>
-      <c r="H51" s="54">
+      <c r="H51" s="41">
         <f>IF(SUM($V51:$AA51), ROUND(AA51/SUM($V51:$AA51), 2),0)</f>
         <v/>
       </c>
@@ -10017,27 +10021,27 @@
       <c r="B52" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="C52" s="54">
+      <c r="C52" s="41">
         <f>IF(SUM($V52:$AA52), ROUND(V52/SUM($V52:$AA52), 2),0)</f>
         <v/>
       </c>
-      <c r="D52" s="54">
+      <c r="D52" s="41">
         <f>IF(SUM($V52:$AA52), ROUND(W52/SUM($V52:$AA52), 2),0)</f>
         <v/>
       </c>
-      <c r="E52" s="54">
+      <c r="E52" s="41">
         <f>IF(SUM($V52:$AA52), ROUND(X52/SUM($V52:$AA52), 2),0)</f>
         <v/>
       </c>
-      <c r="F52" s="54">
+      <c r="F52" s="41">
         <f>IF(SUM($V52:$AA52), ROUND(Y52/SUM($V52:$AA52), 2),0)</f>
         <v/>
       </c>
-      <c r="G52" s="54">
+      <c r="G52" s="41">
         <f>IF(SUM($V52:$AA52), ROUND(Z52/SUM($V52:$AA52), 2),0)</f>
         <v/>
       </c>
-      <c r="H52" s="54">
+      <c r="H52" s="41">
         <f>IF(SUM($V52:$AA52), ROUND(AA52/SUM($V52:$AA52), 2),0)</f>
         <v/>
       </c>
@@ -10099,27 +10103,27 @@
       <c r="B53" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C53" s="54">
+      <c r="C53" s="41">
         <f>IF(SUM($V53:$AA53), ROUND(V53/SUM($V53:$AA53), 2),0)</f>
         <v/>
       </c>
-      <c r="D53" s="54">
+      <c r="D53" s="41">
         <f>IF(SUM($V53:$AA53), ROUND(W53/SUM($V53:$AA53), 2),0)</f>
         <v/>
       </c>
-      <c r="E53" s="54">
+      <c r="E53" s="41">
         <f>IF(SUM($V53:$AA53), ROUND(X53/SUM($V53:$AA53), 2),0)</f>
         <v/>
       </c>
-      <c r="F53" s="54">
+      <c r="F53" s="41">
         <f>IF(SUM($V53:$AA53), ROUND(Y53/SUM($V53:$AA53), 2),0)</f>
         <v/>
       </c>
-      <c r="G53" s="54">
+      <c r="G53" s="41">
         <f>IF(SUM($V53:$AA53), ROUND(Z53/SUM($V53:$AA53), 2),0)</f>
         <v/>
       </c>
-      <c r="H53" s="54">
+      <c r="H53" s="41">
         <f>IF(SUM($V53:$AA53), ROUND(AA53/SUM($V53:$AA53), 2),0)</f>
         <v/>
       </c>
@@ -10181,27 +10185,27 @@
       <c r="B54" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C54" s="54">
+      <c r="C54" s="41">
         <f>IF(SUM($V54:$AA54), ROUND(V54/SUM($V54:$AA54), 2),0)</f>
         <v/>
       </c>
-      <c r="D54" s="54">
+      <c r="D54" s="41">
         <f>IF(SUM($V54:$AA54), ROUND(W54/SUM($V54:$AA54), 2),0)</f>
         <v/>
       </c>
-      <c r="E54" s="54">
+      <c r="E54" s="41">
         <f>IF(SUM($V54:$AA54), ROUND(X54/SUM($V54:$AA54), 2),0)</f>
         <v/>
       </c>
-      <c r="F54" s="54">
+      <c r="F54" s="41">
         <f>IF(SUM($V54:$AA54), ROUND(Y54/SUM($V54:$AA54), 2),0)</f>
         <v/>
       </c>
-      <c r="G54" s="54">
+      <c r="G54" s="41">
         <f>IF(SUM($V54:$AA54), ROUND(Z54/SUM($V54:$AA54), 2),0)</f>
         <v/>
       </c>
-      <c r="H54" s="54">
+      <c r="H54" s="41">
         <f>IF(SUM($V54:$AA54), ROUND(AA54/SUM($V54:$AA54), 2),0)</f>
         <v/>
       </c>
@@ -10263,27 +10267,27 @@
       <c r="B55" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C55" s="54">
+      <c r="C55" s="41">
         <f>IF(SUM($V55:$AA55), ROUND(V55/SUM($V55:$AA55), 2),0)</f>
         <v/>
       </c>
-      <c r="D55" s="54">
+      <c r="D55" s="41">
         <f>IF(SUM($V55:$AA55), ROUND(W55/SUM($V55:$AA55), 2),0)</f>
         <v/>
       </c>
-      <c r="E55" s="54">
+      <c r="E55" s="41">
         <f>IF(SUM($V55:$AA55), ROUND(X55/SUM($V55:$AA55), 2),0)</f>
         <v/>
       </c>
-      <c r="F55" s="54">
+      <c r="F55" s="41">
         <f>IF(SUM($V55:$AA55), ROUND(Y55/SUM($V55:$AA55), 2),0)</f>
         <v/>
       </c>
-      <c r="G55" s="54">
+      <c r="G55" s="41">
         <f>IF(SUM($V55:$AA55), ROUND(Z55/SUM($V55:$AA55), 2),0)</f>
         <v/>
       </c>
-      <c r="H55" s="54">
+      <c r="H55" s="41">
         <f>IF(SUM($V55:$AA55), ROUND(AA55/SUM($V55:$AA55), 2),0)</f>
         <v/>
       </c>
@@ -10345,27 +10349,27 @@
       <c r="B56" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C56" s="54">
+      <c r="C56" s="41">
         <f>IF(SUM($V56:$AA56), ROUND(V56/SUM($V56:$AA56), 2),0)</f>
         <v/>
       </c>
-      <c r="D56" s="54">
+      <c r="D56" s="41">
         <f>IF(SUM($V56:$AA56), ROUND(W56/SUM($V56:$AA56), 2),0)</f>
         <v/>
       </c>
-      <c r="E56" s="54">
+      <c r="E56" s="41">
         <f>IF(SUM($V56:$AA56), ROUND(X56/SUM($V56:$AA56), 2),0)</f>
         <v/>
       </c>
-      <c r="F56" s="54">
+      <c r="F56" s="41">
         <f>IF(SUM($V56:$AA56), ROUND(Y56/SUM($V56:$AA56), 2),0)</f>
         <v/>
       </c>
-      <c r="G56" s="54">
+      <c r="G56" s="41">
         <f>IF(SUM($V56:$AA56), ROUND(Z56/SUM($V56:$AA56), 2),0)</f>
         <v/>
       </c>
-      <c r="H56" s="54">
+      <c r="H56" s="41">
         <f>IF(SUM($V56:$AA56), ROUND(AA56/SUM($V56:$AA56), 2),0)</f>
         <v/>
       </c>
@@ -10427,27 +10431,27 @@
       <c r="B57" s="26" t="n">
         <v>23</v>
       </c>
-      <c r="C57" s="54">
+      <c r="C57" s="41">
         <f>IF(SUM($V57:$AA57), ROUND(V57/SUM($V57:$AA57), 2),0)</f>
         <v/>
       </c>
-      <c r="D57" s="54">
+      <c r="D57" s="41">
         <f>IF(SUM($V57:$AA57), ROUND(W57/SUM($V57:$AA57), 2),0)</f>
         <v/>
       </c>
-      <c r="E57" s="54">
+      <c r="E57" s="41">
         <f>IF(SUM($V57:$AA57), ROUND(X57/SUM($V57:$AA57), 2),0)</f>
         <v/>
       </c>
-      <c r="F57" s="54">
+      <c r="F57" s="41">
         <f>IF(SUM($V57:$AA57), ROUND(Y57/SUM($V57:$AA57), 2),0)</f>
         <v/>
       </c>
-      <c r="G57" s="54">
+      <c r="G57" s="41">
         <f>IF(SUM($V57:$AA57), ROUND(Z57/SUM($V57:$AA57), 2),0)</f>
         <v/>
       </c>
-      <c r="H57" s="54">
+      <c r="H57" s="41">
         <f>IF(SUM($V57:$AA57), ROUND(AA57/SUM($V57:$AA57), 2),0)</f>
         <v/>
       </c>
@@ -10509,27 +10513,27 @@
       <c r="B58" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C58" s="54">
+      <c r="C58" s="41">
         <f>IF(SUM($V58:$AA58), ROUND(V58/SUM($V58:$AA58), 2),0)</f>
         <v/>
       </c>
-      <c r="D58" s="54">
+      <c r="D58" s="41">
         <f>IF(SUM($V58:$AA58), ROUND(W58/SUM($V58:$AA58), 2),0)</f>
         <v/>
       </c>
-      <c r="E58" s="54">
+      <c r="E58" s="41">
         <f>IF(SUM($V58:$AA58), ROUND(X58/SUM($V58:$AA58), 2),0)</f>
         <v/>
       </c>
-      <c r="F58" s="54">
+      <c r="F58" s="41">
         <f>IF(SUM($V58:$AA58), ROUND(Y58/SUM($V58:$AA58), 2),0)</f>
         <v/>
       </c>
-      <c r="G58" s="54">
+      <c r="G58" s="41">
         <f>IF(SUM($V58:$AA58), ROUND(Z58/SUM($V58:$AA58), 2),0)</f>
         <v/>
       </c>
-      <c r="H58" s="54">
+      <c r="H58" s="41">
         <f>IF(SUM($V58:$AA58), ROUND(AA58/SUM($V58:$AA58), 2),0)</f>
         <v/>
       </c>
@@ -10591,27 +10595,27 @@
       <c r="B59" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C59" s="54">
+      <c r="C59" s="41">
         <f>IF(SUM($V59:$AA59), ROUND(V59/SUM($V59:$AA59), 2),0)</f>
         <v/>
       </c>
-      <c r="D59" s="54">
+      <c r="D59" s="41">
         <f>IF(SUM($V59:$AA59), ROUND(W59/SUM($V59:$AA59), 2),0)</f>
         <v/>
       </c>
-      <c r="E59" s="54">
+      <c r="E59" s="41">
         <f>IF(SUM($V59:$AA59), ROUND(X59/SUM($V59:$AA59), 2),0)</f>
         <v/>
       </c>
-      <c r="F59" s="54">
+      <c r="F59" s="41">
         <f>IF(SUM($V59:$AA59), ROUND(Y59/SUM($V59:$AA59), 2),0)</f>
         <v/>
       </c>
-      <c r="G59" s="54">
+      <c r="G59" s="41">
         <f>IF(SUM($V59:$AA59), ROUND(Z59/SUM($V59:$AA59), 2),0)</f>
         <v/>
       </c>
-      <c r="H59" s="54">
+      <c r="H59" s="41">
         <f>IF(SUM($V59:$AA59), ROUND(AA59/SUM($V59:$AA59), 2),0)</f>
         <v/>
       </c>
@@ -10673,27 +10677,27 @@
       <c r="B60" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C60" s="54">
+      <c r="C60" s="41">
         <f>IF(SUM($V60:$AA60), ROUND(V60/SUM($V60:$AA60), 2),0)</f>
         <v/>
       </c>
-      <c r="D60" s="54">
+      <c r="D60" s="41">
         <f>IF(SUM($V60:$AA60), ROUND(W60/SUM($V60:$AA60), 2),0)</f>
         <v/>
       </c>
-      <c r="E60" s="54">
+      <c r="E60" s="41">
         <f>IF(SUM($V60:$AA60), ROUND(X60/SUM($V60:$AA60), 2),0)</f>
         <v/>
       </c>
-      <c r="F60" s="54">
+      <c r="F60" s="41">
         <f>IF(SUM($V60:$AA60), ROUND(Y60/SUM($V60:$AA60), 2),0)</f>
         <v/>
       </c>
-      <c r="G60" s="54">
+      <c r="G60" s="41">
         <f>IF(SUM($V60:$AA60), ROUND(Z60/SUM($V60:$AA60), 2),0)</f>
         <v/>
       </c>
-      <c r="H60" s="54">
+      <c r="H60" s="41">
         <f>IF(SUM($V60:$AA60), ROUND(AA60/SUM($V60:$AA60), 2),0)</f>
         <v/>
       </c>
@@ -10755,27 +10759,27 @@
       <c r="B61" s="26" t="n">
         <v>43</v>
       </c>
-      <c r="C61" s="54">
+      <c r="C61" s="41">
         <f>IF(SUM($V61:$AA61), ROUND(V61/SUM($V61:$AA61), 2),0)</f>
         <v/>
       </c>
-      <c r="D61" s="54">
+      <c r="D61" s="41">
         <f>IF(SUM($V61:$AA61), ROUND(W61/SUM($V61:$AA61), 2),0)</f>
         <v/>
       </c>
-      <c r="E61" s="54">
+      <c r="E61" s="41">
         <f>IF(SUM($V61:$AA61), ROUND(X61/SUM($V61:$AA61), 2),0)</f>
         <v/>
       </c>
-      <c r="F61" s="54">
+      <c r="F61" s="41">
         <f>IF(SUM($V61:$AA61), ROUND(Y61/SUM($V61:$AA61), 2),0)</f>
         <v/>
       </c>
-      <c r="G61" s="54">
+      <c r="G61" s="41">
         <f>IF(SUM($V61:$AA61), ROUND(Z61/SUM($V61:$AA61), 2),0)</f>
         <v/>
       </c>
-      <c r="H61" s="54">
+      <c r="H61" s="41">
         <f>IF(SUM($V61:$AA61), ROUND(AA61/SUM($V61:$AA61), 2),0)</f>
         <v/>
       </c>
@@ -10837,27 +10841,27 @@
       <c r="B62" s="26" t="n">
         <v>44</v>
       </c>
-      <c r="C62" s="54">
+      <c r="C62" s="41">
         <f>IF(SUM($V62:$AA62), ROUND(V62/SUM($V62:$AA62), 2),0)</f>
         <v/>
       </c>
-      <c r="D62" s="54">
+      <c r="D62" s="41">
         <f>IF(SUM($V62:$AA62), ROUND(W62/SUM($V62:$AA62), 2),0)</f>
         <v/>
       </c>
-      <c r="E62" s="54">
+      <c r="E62" s="41">
         <f>IF(SUM($V62:$AA62), ROUND(X62/SUM($V62:$AA62), 2),0)</f>
         <v/>
       </c>
-      <c r="F62" s="54">
+      <c r="F62" s="41">
         <f>IF(SUM($V62:$AA62), ROUND(Y62/SUM($V62:$AA62), 2),0)</f>
         <v/>
       </c>
-      <c r="G62" s="54">
+      <c r="G62" s="41">
         <f>IF(SUM($V62:$AA62), ROUND(Z62/SUM($V62:$AA62), 2),0)</f>
         <v/>
       </c>
-      <c r="H62" s="54">
+      <c r="H62" s="41">
         <f>IF(SUM($V62:$AA62), ROUND(AA62/SUM($V62:$AA62), 2),0)</f>
         <v/>
       </c>
@@ -10919,27 +10923,27 @@
       <c r="B63" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C63" s="54">
+      <c r="C63" s="41">
         <f>IF(SUM($V63:$AA63), ROUND(V63/SUM($V63:$AA63), 2),0)</f>
         <v/>
       </c>
-      <c r="D63" s="54">
+      <c r="D63" s="41">
         <f>IF(SUM($V63:$AA63), ROUND(W63/SUM($V63:$AA63), 2),0)</f>
         <v/>
       </c>
-      <c r="E63" s="54">
+      <c r="E63" s="41">
         <f>IF(SUM($V63:$AA63), ROUND(X63/SUM($V63:$AA63), 2),0)</f>
         <v/>
       </c>
-      <c r="F63" s="54">
+      <c r="F63" s="41">
         <f>IF(SUM($V63:$AA63), ROUND(Y63/SUM($V63:$AA63), 2),0)</f>
         <v/>
       </c>
-      <c r="G63" s="54">
+      <c r="G63" s="41">
         <f>IF(SUM($V63:$AA63), ROUND(Z63/SUM($V63:$AA63), 2),0)</f>
         <v/>
       </c>
-      <c r="H63" s="54">
+      <c r="H63" s="41">
         <f>IF(SUM($V63:$AA63), ROUND(AA63/SUM($V63:$AA63), 2),0)</f>
         <v/>
       </c>
@@ -11001,27 +11005,27 @@
       <c r="B64" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C64" s="54">
+      <c r="C64" s="41">
         <f>IF(SUM($V64:$AA64), ROUND(V64/SUM($V64:$AA64), 2),0)</f>
         <v/>
       </c>
-      <c r="D64" s="54">
+      <c r="D64" s="41">
         <f>IF(SUM($V64:$AA64), ROUND(W64/SUM($V64:$AA64), 2),0)</f>
         <v/>
       </c>
-      <c r="E64" s="54">
+      <c r="E64" s="41">
         <f>IF(SUM($V64:$AA64), ROUND(X64/SUM($V64:$AA64), 2),0)</f>
         <v/>
       </c>
-      <c r="F64" s="54">
+      <c r="F64" s="41">
         <f>IF(SUM($V64:$AA64), ROUND(Y64/SUM($V64:$AA64), 2),0)</f>
         <v/>
       </c>
-      <c r="G64" s="54">
+      <c r="G64" s="41">
         <f>IF(SUM($V64:$AA64), ROUND(Z64/SUM($V64:$AA64), 2),0)</f>
         <v/>
       </c>
-      <c r="H64" s="54">
+      <c r="H64" s="41">
         <f>IF(SUM($V64:$AA64), ROUND(AA64/SUM($V64:$AA64), 2),0)</f>
         <v/>
       </c>
@@ -11083,27 +11087,27 @@
       <c r="B65" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C65" s="54">
+      <c r="C65" s="41">
         <f>IF(SUM($V65:$AA65), ROUND(V65/SUM($V65:$AA65), 2),0)</f>
         <v/>
       </c>
-      <c r="D65" s="54">
+      <c r="D65" s="41">
         <f>IF(SUM($V65:$AA65), ROUND(W65/SUM($V65:$AA65), 2),0)</f>
         <v/>
       </c>
-      <c r="E65" s="54">
+      <c r="E65" s="41">
         <f>IF(SUM($V65:$AA65), ROUND(X65/SUM($V65:$AA65), 2),0)</f>
         <v/>
       </c>
-      <c r="F65" s="54">
+      <c r="F65" s="41">
         <f>IF(SUM($V65:$AA65), ROUND(Y65/SUM($V65:$AA65), 2),0)</f>
         <v/>
       </c>
-      <c r="G65" s="54">
+      <c r="G65" s="41">
         <f>IF(SUM($V65:$AA65), ROUND(Z65/SUM($V65:$AA65), 2),0)</f>
         <v/>
       </c>
-      <c r="H65" s="54">
+      <c r="H65" s="41">
         <f>IF(SUM($V65:$AA65), ROUND(AA65/SUM($V65:$AA65), 2),0)</f>
         <v/>
       </c>
@@ -11165,27 +11169,27 @@
       <c r="B66" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C66" s="54">
+      <c r="C66" s="41">
         <f>IF(SUM($V66:$AA66), ROUND(V66/SUM($V66:$AA66), 2),0)</f>
         <v/>
       </c>
-      <c r="D66" s="54">
+      <c r="D66" s="41">
         <f>IF(SUM($V66:$AA66), ROUND(W66/SUM($V66:$AA66), 2),0)</f>
         <v/>
       </c>
-      <c r="E66" s="54">
+      <c r="E66" s="41">
         <f>IF(SUM($V66:$AA66), ROUND(X66/SUM($V66:$AA66), 2),0)</f>
         <v/>
       </c>
-      <c r="F66" s="54">
+      <c r="F66" s="41">
         <f>IF(SUM($V66:$AA66), ROUND(Y66/SUM($V66:$AA66), 2),0)</f>
         <v/>
       </c>
-      <c r="G66" s="54">
+      <c r="G66" s="41">
         <f>IF(SUM($V66:$AA66), ROUND(Z66/SUM($V66:$AA66), 2),0)</f>
         <v/>
       </c>
-      <c r="H66" s="54">
+      <c r="H66" s="41">
         <f>IF(SUM($V66:$AA66), ROUND(AA66/SUM($V66:$AA66), 2),0)</f>
         <v/>
       </c>
@@ -11247,27 +11251,27 @@
       <c r="B67" s="26" t="n">
         <v>24</v>
       </c>
-      <c r="C67" s="54">
+      <c r="C67" s="41">
         <f>IF(SUM($V67:$AA67), ROUND(V67/SUM($V67:$AA67), 2),0)</f>
         <v/>
       </c>
-      <c r="D67" s="54">
+      <c r="D67" s="41">
         <f>IF(SUM($V67:$AA67), ROUND(W67/SUM($V67:$AA67), 2),0)</f>
         <v/>
       </c>
-      <c r="E67" s="54">
+      <c r="E67" s="41">
         <f>IF(SUM($V67:$AA67), ROUND(X67/SUM($V67:$AA67), 2),0)</f>
         <v/>
       </c>
-      <c r="F67" s="54">
+      <c r="F67" s="41">
         <f>IF(SUM($V67:$AA67), ROUND(Y67/SUM($V67:$AA67), 2),0)</f>
         <v/>
       </c>
-      <c r="G67" s="54">
+      <c r="G67" s="41">
         <f>IF(SUM($V67:$AA67), ROUND(Z67/SUM($V67:$AA67), 2),0)</f>
         <v/>
       </c>
-      <c r="H67" s="54">
+      <c r="H67" s="41">
         <f>IF(SUM($V67:$AA67), ROUND(AA67/SUM($V67:$AA67), 2),0)</f>
         <v/>
       </c>
@@ -11329,27 +11333,27 @@
       <c r="B68" s="26" t="n">
         <v>39</v>
       </c>
-      <c r="C68" s="54">
+      <c r="C68" s="41">
         <f>IF(SUM($V68:$AA68), ROUND(V68/SUM($V68:$AA68), 2),0)</f>
         <v/>
       </c>
-      <c r="D68" s="54">
+      <c r="D68" s="41">
         <f>IF(SUM($V68:$AA68), ROUND(W68/SUM($V68:$AA68), 2),0)</f>
         <v/>
       </c>
-      <c r="E68" s="54">
+      <c r="E68" s="41">
         <f>IF(SUM($V68:$AA68), ROUND(X68/SUM($V68:$AA68), 2),0)</f>
         <v/>
       </c>
-      <c r="F68" s="54">
+      <c r="F68" s="41">
         <f>IF(SUM($V68:$AA68), ROUND(Y68/SUM($V68:$AA68), 2),0)</f>
         <v/>
       </c>
-      <c r="G68" s="54">
+      <c r="G68" s="41">
         <f>IF(SUM($V68:$AA68), ROUND(Z68/SUM($V68:$AA68), 2),0)</f>
         <v/>
       </c>
-      <c r="H68" s="54">
+      <c r="H68" s="41">
         <f>IF(SUM($V68:$AA68), ROUND(AA68/SUM($V68:$AA68), 2),0)</f>
         <v/>
       </c>
@@ -11411,27 +11415,27 @@
       <c r="B69" s="26" t="n">
         <v>36</v>
       </c>
-      <c r="C69" s="54">
+      <c r="C69" s="41">
         <f>IF(SUM($V69:$AA69), ROUND(V69/SUM($V69:$AA69), 2),0)</f>
         <v/>
       </c>
-      <c r="D69" s="54">
+      <c r="D69" s="41">
         <f>IF(SUM($V69:$AA69), ROUND(W69/SUM($V69:$AA69), 2),0)</f>
         <v/>
       </c>
-      <c r="E69" s="54">
+      <c r="E69" s="41">
         <f>IF(SUM($V69:$AA69), ROUND(X69/SUM($V69:$AA69), 2),0)</f>
         <v/>
       </c>
-      <c r="F69" s="54">
+      <c r="F69" s="41">
         <f>IF(SUM($V69:$AA69), ROUND(Y69/SUM($V69:$AA69), 2),0)</f>
         <v/>
       </c>
-      <c r="G69" s="54">
+      <c r="G69" s="41">
         <f>IF(SUM($V69:$AA69), ROUND(Z69/SUM($V69:$AA69), 2),0)</f>
         <v/>
       </c>
-      <c r="H69" s="54">
+      <c r="H69" s="41">
         <f>IF(SUM($V69:$AA69), ROUND(AA69/SUM($V69:$AA69), 2),0)</f>
         <v/>
       </c>
@@ -11493,27 +11497,27 @@
       <c r="B70" s="26" t="n">
         <v>33</v>
       </c>
-      <c r="C70" s="54">
+      <c r="C70" s="41">
         <f>IF(SUM($V70:$AA70), ROUND(V70/SUM($V70:$AA70), 2),0)</f>
         <v/>
       </c>
-      <c r="D70" s="54">
+      <c r="D70" s="41">
         <f>IF(SUM($V70:$AA70), ROUND(W70/SUM($V70:$AA70), 2),0)</f>
         <v/>
       </c>
-      <c r="E70" s="54">
+      <c r="E70" s="41">
         <f>IF(SUM($V70:$AA70), ROUND(X70/SUM($V70:$AA70), 2),0)</f>
         <v/>
       </c>
-      <c r="F70" s="54">
+      <c r="F70" s="41">
         <f>IF(SUM($V70:$AA70), ROUND(Y70/SUM($V70:$AA70), 2),0)</f>
         <v/>
       </c>
-      <c r="G70" s="54">
+      <c r="G70" s="41">
         <f>IF(SUM($V70:$AA70), ROUND(Z70/SUM($V70:$AA70), 2),0)</f>
         <v/>
       </c>
-      <c r="H70" s="54">
+      <c r="H70" s="41">
         <f>IF(SUM($V70:$AA70), ROUND(AA70/SUM($V70:$AA70), 2),0)</f>
         <v/>
       </c>
@@ -11575,27 +11579,27 @@
       <c r="B71" s="26" t="n">
         <v>328</v>
       </c>
-      <c r="C71" s="54">
+      <c r="C71" s="41">
         <f>IF(SUM($V71:$AA71), ROUND(V71/SUM($V71:$AA71), 2),0)</f>
         <v/>
       </c>
-      <c r="D71" s="54">
+      <c r="D71" s="41">
         <f>IF(SUM($V71:$AA71), ROUND(W71/SUM($V71:$AA71), 2),0)</f>
         <v/>
       </c>
-      <c r="E71" s="54">
+      <c r="E71" s="41">
         <f>IF(SUM($V71:$AA71), ROUND(X71/SUM($V71:$AA71), 2),0)</f>
         <v/>
       </c>
-      <c r="F71" s="54">
+      <c r="F71" s="41">
         <f>IF(SUM($V71:$AA71), ROUND(Y71/SUM($V71:$AA71), 2),0)</f>
         <v/>
       </c>
-      <c r="G71" s="54">
+      <c r="G71" s="41">
         <f>IF(SUM($V71:$AA71), ROUND(Z71/SUM($V71:$AA71), 2),0)</f>
         <v/>
       </c>
-      <c r="H71" s="54">
+      <c r="H71" s="41">
         <f>IF(SUM($V71:$AA71), ROUND(AA71/SUM($V71:$AA71), 2),0)</f>
         <v/>
       </c>
@@ -11659,27 +11663,27 @@
       <c r="B72" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C72" s="54">
+      <c r="C72" s="41">
         <f>IF(SUM($V72:$AA72), ROUND(V72/SUM($V72:$AA72), 2),0)</f>
         <v/>
       </c>
-      <c r="D72" s="54">
+      <c r="D72" s="41">
         <f>IF(SUM($V72:$AA72), ROUND(W72/SUM($V72:$AA72), 2),0)</f>
         <v/>
       </c>
-      <c r="E72" s="54">
+      <c r="E72" s="41">
         <f>IF(SUM($V72:$AA72), ROUND(X72/SUM($V72:$AA72), 2),0)</f>
         <v/>
       </c>
-      <c r="F72" s="54">
+      <c r="F72" s="41">
         <f>IF(SUM($V72:$AA72), ROUND(Y72/SUM($V72:$AA72), 2),0)</f>
         <v/>
       </c>
-      <c r="G72" s="54">
+      <c r="G72" s="41">
         <f>IF(SUM($V72:$AA72), ROUND(Z72/SUM($V72:$AA72), 2),0)</f>
         <v/>
       </c>
-      <c r="H72" s="54">
+      <c r="H72" s="41">
         <f>IF(SUM($V72:$AA72), ROUND(AA72/SUM($V72:$AA72), 2),0)</f>
         <v/>
       </c>
@@ -11741,27 +11745,27 @@
       <c r="B73" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C73" s="54">
+      <c r="C73" s="41">
         <f>IF(SUM($V73:$AA73), ROUND(V73/SUM($V73:$AA73), 2),0)</f>
         <v/>
       </c>
-      <c r="D73" s="54">
+      <c r="D73" s="41">
         <f>IF(SUM($V73:$AA73), ROUND(W73/SUM($V73:$AA73), 2),0)</f>
         <v/>
       </c>
-      <c r="E73" s="54">
+      <c r="E73" s="41">
         <f>IF(SUM($V73:$AA73), ROUND(X73/SUM($V73:$AA73), 2),0)</f>
         <v/>
       </c>
-      <c r="F73" s="54">
+      <c r="F73" s="41">
         <f>IF(SUM($V73:$AA73), ROUND(Y73/SUM($V73:$AA73), 2),0)</f>
         <v/>
       </c>
-      <c r="G73" s="54">
+      <c r="G73" s="41">
         <f>IF(SUM($V73:$AA73), ROUND(Z73/SUM($V73:$AA73), 2),0)</f>
         <v/>
       </c>
-      <c r="H73" s="54">
+      <c r="H73" s="41">
         <f>IF(SUM($V73:$AA73), ROUND(AA73/SUM($V73:$AA73), 2),0)</f>
         <v/>
       </c>
@@ -11823,27 +11827,27 @@
       <c r="B74" s="26" t="n">
         <v>31</v>
       </c>
-      <c r="C74" s="54">
+      <c r="C74" s="41">
         <f>IF(SUM($V74:$AA74), ROUND(V74/SUM($V74:$AA74), 2),0)</f>
         <v/>
       </c>
-      <c r="D74" s="54">
+      <c r="D74" s="41">
         <f>IF(SUM($V74:$AA74), ROUND(W74/SUM($V74:$AA74), 2),0)</f>
         <v/>
       </c>
-      <c r="E74" s="54">
+      <c r="E74" s="41">
         <f>IF(SUM($V74:$AA74), ROUND(X74/SUM($V74:$AA74), 2),0)</f>
         <v/>
       </c>
-      <c r="F74" s="54">
+      <c r="F74" s="41">
         <f>IF(SUM($V74:$AA74), ROUND(Y74/SUM($V74:$AA74), 2),0)</f>
         <v/>
       </c>
-      <c r="G74" s="54">
+      <c r="G74" s="41">
         <f>IF(SUM($V74:$AA74), ROUND(Z74/SUM($V74:$AA74), 2),0)</f>
         <v/>
       </c>
-      <c r="H74" s="54">
+      <c r="H74" s="41">
         <f>IF(SUM($V74:$AA74), ROUND(AA74/SUM($V74:$AA74), 2),0)</f>
         <v/>
       </c>
@@ -11905,27 +11909,27 @@
       <c r="B75" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C75" s="54">
+      <c r="C75" s="41">
         <f>IF(SUM($V75:$AA75), ROUND(V75/SUM($V75:$AA75), 2),0)</f>
         <v/>
       </c>
-      <c r="D75" s="54">
+      <c r="D75" s="41">
         <f>IF(SUM($V75:$AA75), ROUND(W75/SUM($V75:$AA75), 2),0)</f>
         <v/>
       </c>
-      <c r="E75" s="54">
+      <c r="E75" s="41">
         <f>IF(SUM($V75:$AA75), ROUND(X75/SUM($V75:$AA75), 2),0)</f>
         <v/>
       </c>
-      <c r="F75" s="54">
+      <c r="F75" s="41">
         <f>IF(SUM($V75:$AA75), ROUND(Y75/SUM($V75:$AA75), 2),0)</f>
         <v/>
       </c>
-      <c r="G75" s="54">
+      <c r="G75" s="41">
         <f>IF(SUM($V75:$AA75), ROUND(Z75/SUM($V75:$AA75), 2),0)</f>
         <v/>
       </c>
-      <c r="H75" s="54">
+      <c r="H75" s="41">
         <f>IF(SUM($V75:$AA75), ROUND(AA75/SUM($V75:$AA75), 2),0)</f>
         <v/>
       </c>
@@ -11987,27 +11991,27 @@
       <c r="B76" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C76" s="54">
+      <c r="C76" s="41">
         <f>IF(SUM($V76:$AA76), ROUND(V76/SUM($V76:$AA76), 2),0)</f>
         <v/>
       </c>
-      <c r="D76" s="54">
+      <c r="D76" s="41">
         <f>IF(SUM($V76:$AA76), ROUND(W76/SUM($V76:$AA76), 2),0)</f>
         <v/>
       </c>
-      <c r="E76" s="54">
+      <c r="E76" s="41">
         <f>IF(SUM($V76:$AA76), ROUND(X76/SUM($V76:$AA76), 2),0)</f>
         <v/>
       </c>
-      <c r="F76" s="54">
+      <c r="F76" s="41">
         <f>IF(SUM($V76:$AA76), ROUND(Y76/SUM($V76:$AA76), 2),0)</f>
         <v/>
       </c>
-      <c r="G76" s="54">
+      <c r="G76" s="41">
         <f>IF(SUM($V76:$AA76), ROUND(Z76/SUM($V76:$AA76), 2),0)</f>
         <v/>
       </c>
-      <c r="H76" s="54">
+      <c r="H76" s="41">
         <f>IF(SUM($V76:$AA76), ROUND(AA76/SUM($V76:$AA76), 2),0)</f>
         <v/>
       </c>
@@ -12069,27 +12073,27 @@
       <c r="B77" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C77" s="54">
+      <c r="C77" s="41">
         <f>IF(SUM($V77:$AA77), ROUND(V77/SUM($V77:$AA77), 2),0)</f>
         <v/>
       </c>
-      <c r="D77" s="54">
+      <c r="D77" s="41">
         <f>IF(SUM($V77:$AA77), ROUND(W77/SUM($V77:$AA77), 2),0)</f>
         <v/>
       </c>
-      <c r="E77" s="54">
+      <c r="E77" s="41">
         <f>IF(SUM($V77:$AA77), ROUND(X77/SUM($V77:$AA77), 2),0)</f>
         <v/>
       </c>
-      <c r="F77" s="54">
+      <c r="F77" s="41">
         <f>IF(SUM($V77:$AA77), ROUND(Y77/SUM($V77:$AA77), 2),0)</f>
         <v/>
       </c>
-      <c r="G77" s="54">
+      <c r="G77" s="41">
         <f>IF(SUM($V77:$AA77), ROUND(Z77/SUM($V77:$AA77), 2),0)</f>
         <v/>
       </c>
-      <c r="H77" s="54">
+      <c r="H77" s="41">
         <f>IF(SUM($V77:$AA77), ROUND(AA77/SUM($V77:$AA77), 2),0)</f>
         <v/>
       </c>
@@ -12151,27 +12155,27 @@
       <c r="B78" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C78" s="54">
+      <c r="C78" s="41">
         <f>IF(SUM($V78:$AA78), ROUND(V78/SUM($V78:$AA78), 2),0)</f>
         <v/>
       </c>
-      <c r="D78" s="54">
+      <c r="D78" s="41">
         <f>IF(SUM($V78:$AA78), ROUND(W78/SUM($V78:$AA78), 2),0)</f>
         <v/>
       </c>
-      <c r="E78" s="54">
+      <c r="E78" s="41">
         <f>IF(SUM($V78:$AA78), ROUND(X78/SUM($V78:$AA78), 2),0)</f>
         <v/>
       </c>
-      <c r="F78" s="54">
+      <c r="F78" s="41">
         <f>IF(SUM($V78:$AA78), ROUND(Y78/SUM($V78:$AA78), 2),0)</f>
         <v/>
       </c>
-      <c r="G78" s="54">
+      <c r="G78" s="41">
         <f>IF(SUM($V78:$AA78), ROUND(Z78/SUM($V78:$AA78), 2),0)</f>
         <v/>
       </c>
-      <c r="H78" s="54">
+      <c r="H78" s="41">
         <f>IF(SUM($V78:$AA78), ROUND(AA78/SUM($V78:$AA78), 2),0)</f>
         <v/>
       </c>
@@ -12233,27 +12237,27 @@
       <c r="B79" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="C79" s="54">
+      <c r="C79" s="41">
         <f>IF(SUM($V79:$AA79), ROUND(V79/SUM($V79:$AA79), 2),0)</f>
         <v/>
       </c>
-      <c r="D79" s="54">
+      <c r="D79" s="41">
         <f>IF(SUM($V79:$AA79), ROUND(W79/SUM($V79:$AA79), 2),0)</f>
         <v/>
       </c>
-      <c r="E79" s="54">
+      <c r="E79" s="41">
         <f>IF(SUM($V79:$AA79), ROUND(X79/SUM($V79:$AA79), 2),0)</f>
         <v/>
       </c>
-      <c r="F79" s="54">
+      <c r="F79" s="41">
         <f>IF(SUM($V79:$AA79), ROUND(Y79/SUM($V79:$AA79), 2),0)</f>
         <v/>
       </c>
-      <c r="G79" s="54">
+      <c r="G79" s="41">
         <f>IF(SUM($V79:$AA79), ROUND(Z79/SUM($V79:$AA79), 2),0)</f>
         <v/>
       </c>
-      <c r="H79" s="54">
+      <c r="H79" s="41">
         <f>IF(SUM($V79:$AA79), ROUND(AA79/SUM($V79:$AA79), 2),0)</f>
         <v/>
       </c>
@@ -12315,27 +12319,27 @@
       <c r="B80" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C80" s="54">
+      <c r="C80" s="41">
         <f>IF(SUM($V80:$AA80), ROUND(V80/SUM($V80:$AA80), 2),0)</f>
         <v/>
       </c>
-      <c r="D80" s="54">
+      <c r="D80" s="41">
         <f>IF(SUM($V80:$AA80), ROUND(W80/SUM($V80:$AA80), 2),0)</f>
         <v/>
       </c>
-      <c r="E80" s="54">
+      <c r="E80" s="41">
         <f>IF(SUM($V80:$AA80), ROUND(X80/SUM($V80:$AA80), 2),0)</f>
         <v/>
       </c>
-      <c r="F80" s="54">
+      <c r="F80" s="41">
         <f>IF(SUM($V80:$AA80), ROUND(Y80/SUM($V80:$AA80), 2),0)</f>
         <v/>
       </c>
-      <c r="G80" s="54">
+      <c r="G80" s="41">
         <f>IF(SUM($V80:$AA80), ROUND(Z80/SUM($V80:$AA80), 2),0)</f>
         <v/>
       </c>
-      <c r="H80" s="54">
+      <c r="H80" s="41">
         <f>IF(SUM($V80:$AA80), ROUND(AA80/SUM($V80:$AA80), 2),0)</f>
         <v/>
       </c>
@@ -12397,27 +12401,27 @@
       <c r="B81" s="26" t="n">
         <v>109</v>
       </c>
-      <c r="C81" s="54">
+      <c r="C81" s="41">
         <f>IF(SUM($V81:$AA81), ROUND(V81/SUM($V81:$AA81), 2),0)</f>
         <v/>
       </c>
-      <c r="D81" s="54">
+      <c r="D81" s="41">
         <f>IF(SUM($V81:$AA81), ROUND(W81/SUM($V81:$AA81), 2),0)</f>
         <v/>
       </c>
-      <c r="E81" s="54">
+      <c r="E81" s="41">
         <f>IF(SUM($V81:$AA81), ROUND(X81/SUM($V81:$AA81), 2),0)</f>
         <v/>
       </c>
-      <c r="F81" s="54">
+      <c r="F81" s="41">
         <f>IF(SUM($V81:$AA81), ROUND(Y81/SUM($V81:$AA81), 2),0)</f>
         <v/>
       </c>
-      <c r="G81" s="54">
+      <c r="G81" s="41">
         <f>IF(SUM($V81:$AA81), ROUND(Z81/SUM($V81:$AA81), 2),0)</f>
         <v/>
       </c>
-      <c r="H81" s="54">
+      <c r="H81" s="41">
         <f>IF(SUM($V81:$AA81), ROUND(AA81/SUM($V81:$AA81), 2),0)</f>
         <v/>
       </c>
@@ -12479,27 +12483,27 @@
       <c r="B82" s="26" t="n">
         <v>48</v>
       </c>
-      <c r="C82" s="54">
+      <c r="C82" s="41">
         <f>IF(SUM($V82:$AA82), ROUND(V82/SUM($V82:$AA82), 2),0)</f>
         <v/>
       </c>
-      <c r="D82" s="54">
+      <c r="D82" s="41">
         <f>IF(SUM($V82:$AA82), ROUND(W82/SUM($V82:$AA82), 2),0)</f>
         <v/>
       </c>
-      <c r="E82" s="54">
+      <c r="E82" s="41">
         <f>IF(SUM($V82:$AA82), ROUND(X82/SUM($V82:$AA82), 2),0)</f>
         <v/>
       </c>
-      <c r="F82" s="54">
+      <c r="F82" s="41">
         <f>IF(SUM($V82:$AA82), ROUND(Y82/SUM($V82:$AA82), 2),0)</f>
         <v/>
       </c>
-      <c r="G82" s="54">
+      <c r="G82" s="41">
         <f>IF(SUM($V82:$AA82), ROUND(Z82/SUM($V82:$AA82), 2),0)</f>
         <v/>
       </c>
-      <c r="H82" s="54">
+      <c r="H82" s="41">
         <f>IF(SUM($V82:$AA82), ROUND(AA82/SUM($V82:$AA82), 2),0)</f>
         <v/>
       </c>
@@ -12561,27 +12565,27 @@
       <c r="B83" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C83" s="54">
+      <c r="C83" s="41">
         <f>IF(SUM($V83:$AA83), ROUND(V83/SUM($V83:$AA83), 2),0)</f>
         <v/>
       </c>
-      <c r="D83" s="54">
+      <c r="D83" s="41">
         <f>IF(SUM($V83:$AA83), ROUND(W83/SUM($V83:$AA83), 2),0)</f>
         <v/>
       </c>
-      <c r="E83" s="54">
+      <c r="E83" s="41">
         <f>IF(SUM($V83:$AA83), ROUND(X83/SUM($V83:$AA83), 2),0)</f>
         <v/>
       </c>
-      <c r="F83" s="54">
+      <c r="F83" s="41">
         <f>IF(SUM($V83:$AA83), ROUND(Y83/SUM($V83:$AA83), 2),0)</f>
         <v/>
       </c>
-      <c r="G83" s="54">
+      <c r="G83" s="41">
         <f>IF(SUM($V83:$AA83), ROUND(Z83/SUM($V83:$AA83), 2),0)</f>
         <v/>
       </c>
-      <c r="H83" s="54">
+      <c r="H83" s="41">
         <f>IF(SUM($V83:$AA83), ROUND(AA83/SUM($V83:$AA83), 2),0)</f>
         <v/>
       </c>
@@ -12643,27 +12647,27 @@
       <c r="B84" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="C84" s="54">
+      <c r="C84" s="41">
         <f>IF(SUM($V84:$AA84), ROUND(V84/SUM($V84:$AA84), 2),0)</f>
         <v/>
       </c>
-      <c r="D84" s="54">
+      <c r="D84" s="41">
         <f>IF(SUM($V84:$AA84), ROUND(W84/SUM($V84:$AA84), 2),0)</f>
         <v/>
       </c>
-      <c r="E84" s="54">
+      <c r="E84" s="41">
         <f>IF(SUM($V84:$AA84), ROUND(X84/SUM($V84:$AA84), 2),0)</f>
         <v/>
       </c>
-      <c r="F84" s="54">
+      <c r="F84" s="41">
         <f>IF(SUM($V84:$AA84), ROUND(Y84/SUM($V84:$AA84), 2),0)</f>
         <v/>
       </c>
-      <c r="G84" s="54">
+      <c r="G84" s="41">
         <f>IF(SUM($V84:$AA84), ROUND(Z84/SUM($V84:$AA84), 2),0)</f>
         <v/>
       </c>
-      <c r="H84" s="54">
+      <c r="H84" s="41">
         <f>IF(SUM($V84:$AA84), ROUND(AA84/SUM($V84:$AA84), 2),0)</f>
         <v/>
       </c>
@@ -12725,27 +12729,27 @@
       <c r="B85" s="26" t="n">
         <v>43</v>
       </c>
-      <c r="C85" s="54">
+      <c r="C85" s="41">
         <f>IF(SUM($V85:$AA85), ROUND(V85/SUM($V85:$AA85), 2),0)</f>
         <v/>
       </c>
-      <c r="D85" s="54">
+      <c r="D85" s="41">
         <f>IF(SUM($V85:$AA85), ROUND(W85/SUM($V85:$AA85), 2),0)</f>
         <v/>
       </c>
-      <c r="E85" s="54">
+      <c r="E85" s="41">
         <f>IF(SUM($V85:$AA85), ROUND(X85/SUM($V85:$AA85), 2),0)</f>
         <v/>
       </c>
-      <c r="F85" s="54">
+      <c r="F85" s="41">
         <f>IF(SUM($V85:$AA85), ROUND(Y85/SUM($V85:$AA85), 2),0)</f>
         <v/>
       </c>
-      <c r="G85" s="54">
+      <c r="G85" s="41">
         <f>IF(SUM($V85:$AA85), ROUND(Z85/SUM($V85:$AA85), 2),0)</f>
         <v/>
       </c>
-      <c r="H85" s="54">
+      <c r="H85" s="41">
         <f>IF(SUM($V85:$AA85), ROUND(AA85/SUM($V85:$AA85), 2),0)</f>
         <v/>
       </c>
@@ -12807,27 +12811,27 @@
       <c r="B86" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C86" s="54">
+      <c r="C86" s="41">
         <f>IF(SUM($V86:$AA86), ROUND(V86/SUM($V86:$AA86), 2),0)</f>
         <v/>
       </c>
-      <c r="D86" s="54">
+      <c r="D86" s="41">
         <f>IF(SUM($V86:$AA86), ROUND(W86/SUM($V86:$AA86), 2),0)</f>
         <v/>
       </c>
-      <c r="E86" s="54">
+      <c r="E86" s="41">
         <f>IF(SUM($V86:$AA86), ROUND(X86/SUM($V86:$AA86), 2),0)</f>
         <v/>
       </c>
-      <c r="F86" s="54">
+      <c r="F86" s="41">
         <f>IF(SUM($V86:$AA86), ROUND(Y86/SUM($V86:$AA86), 2),0)</f>
         <v/>
       </c>
-      <c r="G86" s="54">
+      <c r="G86" s="41">
         <f>IF(SUM($V86:$AA86), ROUND(Z86/SUM($V86:$AA86), 2),0)</f>
         <v/>
       </c>
-      <c r="H86" s="54">
+      <c r="H86" s="41">
         <f>IF(SUM($V86:$AA86), ROUND(AA86/SUM($V86:$AA86), 2),0)</f>
         <v/>
       </c>
@@ -12889,27 +12893,27 @@
       <c r="B87" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C87" s="54">
+      <c r="C87" s="41">
         <f>IF(SUM($V87:$AA87), ROUND(V87/SUM($V87:$AA87), 2),0)</f>
         <v/>
       </c>
-      <c r="D87" s="54">
+      <c r="D87" s="41">
         <f>IF(SUM($V87:$AA87), ROUND(W87/SUM($V87:$AA87), 2),0)</f>
         <v/>
       </c>
-      <c r="E87" s="54">
+      <c r="E87" s="41">
         <f>IF(SUM($V87:$AA87), ROUND(X87/SUM($V87:$AA87), 2),0)</f>
         <v/>
       </c>
-      <c r="F87" s="54">
+      <c r="F87" s="41">
         <f>IF(SUM($V87:$AA87), ROUND(Y87/SUM($V87:$AA87), 2),0)</f>
         <v/>
       </c>
-      <c r="G87" s="54">
+      <c r="G87" s="41">
         <f>IF(SUM($V87:$AA87), ROUND(Z87/SUM($V87:$AA87), 2),0)</f>
         <v/>
       </c>
-      <c r="H87" s="54">
+      <c r="H87" s="41">
         <f>IF(SUM($V87:$AA87), ROUND(AA87/SUM($V87:$AA87), 2),0)</f>
         <v/>
       </c>
@@ -12971,27 +12975,27 @@
       <c r="B88" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C88" s="54">
+      <c r="C88" s="41">
         <f>IF(SUM($V88:$AA88), ROUND(V88/SUM($V88:$AA88), 2),0)</f>
         <v/>
       </c>
-      <c r="D88" s="54">
+      <c r="D88" s="41">
         <f>IF(SUM($V88:$AA88), ROUND(W88/SUM($V88:$AA88), 2),0)</f>
         <v/>
       </c>
-      <c r="E88" s="54">
+      <c r="E88" s="41">
         <f>IF(SUM($V88:$AA88), ROUND(X88/SUM($V88:$AA88), 2),0)</f>
         <v/>
       </c>
-      <c r="F88" s="54">
+      <c r="F88" s="41">
         <f>IF(SUM($V88:$AA88), ROUND(Y88/SUM($V88:$AA88), 2),0)</f>
         <v/>
       </c>
-      <c r="G88" s="54">
+      <c r="G88" s="41">
         <f>IF(SUM($V88:$AA88), ROUND(Z88/SUM($V88:$AA88), 2),0)</f>
         <v/>
       </c>
-      <c r="H88" s="54">
+      <c r="H88" s="41">
         <f>IF(SUM($V88:$AA88), ROUND(AA88/SUM($V88:$AA88), 2),0)</f>
         <v/>
       </c>
@@ -13053,27 +13057,27 @@
       <c r="B89" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="C89" s="54">
+      <c r="C89" s="41">
         <f>IF(SUM($V89:$AA89), ROUND(V89/SUM($V89:$AA89), 2),0)</f>
         <v/>
       </c>
-      <c r="D89" s="54">
+      <c r="D89" s="41">
         <f>IF(SUM($V89:$AA89), ROUND(W89/SUM($V89:$AA89), 2),0)</f>
         <v/>
       </c>
-      <c r="E89" s="54">
+      <c r="E89" s="41">
         <f>IF(SUM($V89:$AA89), ROUND(X89/SUM($V89:$AA89), 2),0)</f>
         <v/>
       </c>
-      <c r="F89" s="54">
+      <c r="F89" s="41">
         <f>IF(SUM($V89:$AA89), ROUND(Y89/SUM($V89:$AA89), 2),0)</f>
         <v/>
       </c>
-      <c r="G89" s="54">
+      <c r="G89" s="41">
         <f>IF(SUM($V89:$AA89), ROUND(Z89/SUM($V89:$AA89), 2),0)</f>
         <v/>
       </c>
-      <c r="H89" s="54">
+      <c r="H89" s="41">
         <f>IF(SUM($V89:$AA89), ROUND(AA89/SUM($V89:$AA89), 2),0)</f>
         <v/>
       </c>
@@ -13135,27 +13139,27 @@
       <c r="B90" s="26" t="n">
         <v>67</v>
       </c>
-      <c r="C90" s="54">
+      <c r="C90" s="41">
         <f>IF(SUM($V90:$AA90), ROUND(V90/SUM($V90:$AA90), 2),0)</f>
         <v/>
       </c>
-      <c r="D90" s="54">
+      <c r="D90" s="41">
         <f>IF(SUM($V90:$AA90), ROUND(W90/SUM($V90:$AA90), 2),0)</f>
         <v/>
       </c>
-      <c r="E90" s="54">
+      <c r="E90" s="41">
         <f>IF(SUM($V90:$AA90), ROUND(X90/SUM($V90:$AA90), 2),0)</f>
         <v/>
       </c>
-      <c r="F90" s="54">
+      <c r="F90" s="41">
         <f>IF(SUM($V90:$AA90), ROUND(Y90/SUM($V90:$AA90), 2),0)</f>
         <v/>
       </c>
-      <c r="G90" s="54">
+      <c r="G90" s="41">
         <f>IF(SUM($V90:$AA90), ROUND(Z90/SUM($V90:$AA90), 2),0)</f>
         <v/>
       </c>
-      <c r="H90" s="54">
+      <c r="H90" s="41">
         <f>IF(SUM($V90:$AA90), ROUND(AA90/SUM($V90:$AA90), 2),0)</f>
         <v/>
       </c>
@@ -13217,27 +13221,27 @@
       <c r="B91" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="C91" s="54">
+      <c r="C91" s="41">
         <f>IF(SUM($V91:$AA91), ROUND(V91/SUM($V91:$AA91), 2),0)</f>
         <v/>
       </c>
-      <c r="D91" s="54">
+      <c r="D91" s="41">
         <f>IF(SUM($V91:$AA91), ROUND(W91/SUM($V91:$AA91), 2),0)</f>
         <v/>
       </c>
-      <c r="E91" s="54">
+      <c r="E91" s="41">
         <f>IF(SUM($V91:$AA91), ROUND(X91/SUM($V91:$AA91), 2),0)</f>
         <v/>
       </c>
-      <c r="F91" s="54">
+      <c r="F91" s="41">
         <f>IF(SUM($V91:$AA91), ROUND(Y91/SUM($V91:$AA91), 2),0)</f>
         <v/>
       </c>
-      <c r="G91" s="54">
+      <c r="G91" s="41">
         <f>IF(SUM($V91:$AA91), ROUND(Z91/SUM($V91:$AA91), 2),0)</f>
         <v/>
       </c>
-      <c r="H91" s="54">
+      <c r="H91" s="41">
         <f>IF(SUM($V91:$AA91), ROUND(AA91/SUM($V91:$AA91), 2),0)</f>
         <v/>
       </c>
@@ -13299,27 +13303,27 @@
       <c r="B92" s="26" t="n">
         <v>26</v>
       </c>
-      <c r="C92" s="54">
+      <c r="C92" s="41">
         <f>IF(SUM($V92:$AA92), ROUND(V92/SUM($V92:$AA92), 2),0)</f>
         <v/>
       </c>
-      <c r="D92" s="54">
+      <c r="D92" s="41">
         <f>IF(SUM($V92:$AA92), ROUND(W92/SUM($V92:$AA92), 2),0)</f>
         <v/>
       </c>
-      <c r="E92" s="54">
+      <c r="E92" s="41">
         <f>IF(SUM($V92:$AA92), ROUND(X92/SUM($V92:$AA92), 2),0)</f>
         <v/>
       </c>
-      <c r="F92" s="54">
+      <c r="F92" s="41">
         <f>IF(SUM($V92:$AA92), ROUND(Y92/SUM($V92:$AA92), 2),0)</f>
         <v/>
       </c>
-      <c r="G92" s="54">
+      <c r="G92" s="41">
         <f>IF(SUM($V92:$AA92), ROUND(Z92/SUM($V92:$AA92), 2),0)</f>
         <v/>
       </c>
-      <c r="H92" s="54">
+      <c r="H92" s="41">
         <f>IF(SUM($V92:$AA92), ROUND(AA92/SUM($V92:$AA92), 2),0)</f>
         <v/>
       </c>
@@ -13381,27 +13385,27 @@
       <c r="B93" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="C93" s="54">
+      <c r="C93" s="41">
         <f>IF(SUM($V93:$AA93), ROUND(V93/SUM($V93:$AA93), 2),0)</f>
         <v/>
       </c>
-      <c r="D93" s="54">
+      <c r="D93" s="41">
         <f>IF(SUM($V93:$AA93), ROUND(W93/SUM($V93:$AA93), 2),0)</f>
         <v/>
       </c>
-      <c r="E93" s="54">
+      <c r="E93" s="41">
         <f>IF(SUM($V93:$AA93), ROUND(X93/SUM($V93:$AA93), 2),0)</f>
         <v/>
       </c>
-      <c r="F93" s="54">
+      <c r="F93" s="41">
         <f>IF(SUM($V93:$AA93), ROUND(Y93/SUM($V93:$AA93), 2),0)</f>
         <v/>
       </c>
-      <c r="G93" s="54">
+      <c r="G93" s="41">
         <f>IF(SUM($V93:$AA93), ROUND(Z93/SUM($V93:$AA93), 2),0)</f>
         <v/>
       </c>
-      <c r="H93" s="54">
+      <c r="H93" s="41">
         <f>IF(SUM($V93:$AA93), ROUND(AA93/SUM($V93:$AA93), 2),0)</f>
         <v/>
       </c>
@@ -13463,27 +13467,27 @@
       <c r="B94" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="C94" s="54">
+      <c r="C94" s="41">
         <f>IF(SUM($V94:$AA94), ROUND(V94/SUM($V94:$AA94), 2),0)</f>
         <v/>
       </c>
-      <c r="D94" s="54">
+      <c r="D94" s="41">
         <f>IF(SUM($V94:$AA94), ROUND(W94/SUM($V94:$AA94), 2),0)</f>
         <v/>
       </c>
-      <c r="E94" s="54">
+      <c r="E94" s="41">
         <f>IF(SUM($V94:$AA94), ROUND(X94/SUM($V94:$AA94), 2),0)</f>
         <v/>
       </c>
-      <c r="F94" s="54">
+      <c r="F94" s="41">
         <f>IF(SUM($V94:$AA94), ROUND(Y94/SUM($V94:$AA94), 2),0)</f>
         <v/>
       </c>
-      <c r="G94" s="54">
+      <c r="G94" s="41">
         <f>IF(SUM($V94:$AA94), ROUND(Z94/SUM($V94:$AA94), 2),0)</f>
         <v/>
       </c>
-      <c r="H94" s="54">
+      <c r="H94" s="41">
         <f>IF(SUM($V94:$AA94), ROUND(AA94/SUM($V94:$AA94), 2),0)</f>
         <v/>
       </c>
@@ -13545,27 +13549,27 @@
       <c r="B95" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="C95" s="54">
+      <c r="C95" s="41">
         <f>IF(SUM($V95:$AA95), ROUND(V95/SUM($V95:$AA95), 2),0)</f>
         <v/>
       </c>
-      <c r="D95" s="54">
+      <c r="D95" s="41">
         <f>IF(SUM($V95:$AA95), ROUND(W95/SUM($V95:$AA95), 2),0)</f>
         <v/>
       </c>
-      <c r="E95" s="54">
+      <c r="E95" s="41">
         <f>IF(SUM($V95:$AA95), ROUND(X95/SUM($V95:$AA95), 2),0)</f>
         <v/>
       </c>
-      <c r="F95" s="54">
+      <c r="F95" s="41">
         <f>IF(SUM($V95:$AA95), ROUND(Y95/SUM($V95:$AA95), 2),0)</f>
         <v/>
       </c>
-      <c r="G95" s="54">
+      <c r="G95" s="41">
         <f>IF(SUM($V95:$AA95), ROUND(Z95/SUM($V95:$AA95), 2),0)</f>
         <v/>
       </c>
-      <c r="H95" s="54">
+      <c r="H95" s="41">
         <f>IF(SUM($V95:$AA95), ROUND(AA95/SUM($V95:$AA95), 2),0)</f>
         <v/>
       </c>
@@ -13627,27 +13631,27 @@
       <c r="B96" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C96" s="54">
+      <c r="C96" s="41">
         <f>IF(SUM($V96:$AA96), ROUND(V96/SUM($V96:$AA96), 2),0)</f>
         <v/>
       </c>
-      <c r="D96" s="54">
+      <c r="D96" s="41">
         <f>IF(SUM($V96:$AA96), ROUND(W96/SUM($V96:$AA96), 2),0)</f>
         <v/>
       </c>
-      <c r="E96" s="54">
+      <c r="E96" s="41">
         <f>IF(SUM($V96:$AA96), ROUND(X96/SUM($V96:$AA96), 2),0)</f>
         <v/>
       </c>
-      <c r="F96" s="54">
+      <c r="F96" s="41">
         <f>IF(SUM($V96:$AA96), ROUND(Y96/SUM($V96:$AA96), 2),0)</f>
         <v/>
       </c>
-      <c r="G96" s="54">
+      <c r="G96" s="41">
         <f>IF(SUM($V96:$AA96), ROUND(Z96/SUM($V96:$AA96), 2),0)</f>
         <v/>
       </c>
-      <c r="H96" s="54">
+      <c r="H96" s="41">
         <f>IF(SUM($V96:$AA96), ROUND(AA96/SUM($V96:$AA96), 2),0)</f>
         <v/>
       </c>
@@ -13709,27 +13713,27 @@
       <c r="B97" s="26" t="n">
         <v>26</v>
       </c>
-      <c r="C97" s="54">
+      <c r="C97" s="41">
         <f>IF(SUM($V97:$AA97), ROUND(V97/SUM($V97:$AA97), 2),0)</f>
         <v/>
       </c>
-      <c r="D97" s="54">
+      <c r="D97" s="41">
         <f>IF(SUM($V97:$AA97), ROUND(W97/SUM($V97:$AA97), 2),0)</f>
         <v/>
       </c>
-      <c r="E97" s="54">
+      <c r="E97" s="41">
         <f>IF(SUM($V97:$AA97), ROUND(X97/SUM($V97:$AA97), 2),0)</f>
         <v/>
       </c>
-      <c r="F97" s="54">
+      <c r="F97" s="41">
         <f>IF(SUM($V97:$AA97), ROUND(Y97/SUM($V97:$AA97), 2),0)</f>
         <v/>
       </c>
-      <c r="G97" s="54">
+      <c r="G97" s="41">
         <f>IF(SUM($V97:$AA97), ROUND(Z97/SUM($V97:$AA97), 2),0)</f>
         <v/>
       </c>
-      <c r="H97" s="54">
+      <c r="H97" s="41">
         <f>IF(SUM($V97:$AA97), ROUND(AA97/SUM($V97:$AA97), 2),0)</f>
         <v/>
       </c>
@@ -13791,27 +13795,27 @@
       <c r="B98" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C98" s="54">
+      <c r="C98" s="41">
         <f>IF(SUM($V98:$AA98), ROUND(V98/SUM($V98:$AA98), 2),0)</f>
         <v/>
       </c>
-      <c r="D98" s="54">
+      <c r="D98" s="41">
         <f>IF(SUM($V98:$AA98), ROUND(W98/SUM($V98:$AA98), 2),0)</f>
         <v/>
       </c>
-      <c r="E98" s="54">
+      <c r="E98" s="41">
         <f>IF(SUM($V98:$AA98), ROUND(X98/SUM($V98:$AA98), 2),0)</f>
         <v/>
       </c>
-      <c r="F98" s="54">
+      <c r="F98" s="41">
         <f>IF(SUM($V98:$AA98), ROUND(Y98/SUM($V98:$AA98), 2),0)</f>
         <v/>
       </c>
-      <c r="G98" s="54">
+      <c r="G98" s="41">
         <f>IF(SUM($V98:$AA98), ROUND(Z98/SUM($V98:$AA98), 2),0)</f>
         <v/>
       </c>
-      <c r="H98" s="54">
+      <c r="H98" s="41">
         <f>IF(SUM($V98:$AA98), ROUND(AA98/SUM($V98:$AA98), 2),0)</f>
         <v/>
       </c>
@@ -13873,27 +13877,27 @@
       <c r="B99" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C99" s="54">
+      <c r="C99" s="41">
         <f>IF(SUM($V99:$AA99), ROUND(V99/SUM($V99:$AA99), 2),0)</f>
         <v/>
       </c>
-      <c r="D99" s="54">
+      <c r="D99" s="41">
         <f>IF(SUM($V99:$AA99), ROUND(W99/SUM($V99:$AA99), 2),0)</f>
         <v/>
       </c>
-      <c r="E99" s="54">
+      <c r="E99" s="41">
         <f>IF(SUM($V99:$AA99), ROUND(X99/SUM($V99:$AA99), 2),0)</f>
         <v/>
       </c>
-      <c r="F99" s="54">
+      <c r="F99" s="41">
         <f>IF(SUM($V99:$AA99), ROUND(Y99/SUM($V99:$AA99), 2),0)</f>
         <v/>
       </c>
-      <c r="G99" s="54">
+      <c r="G99" s="41">
         <f>IF(SUM($V99:$AA99), ROUND(Z99/SUM($V99:$AA99), 2),0)</f>
         <v/>
       </c>
-      <c r="H99" s="54">
+      <c r="H99" s="41">
         <f>IF(SUM($V99:$AA99), ROUND(AA99/SUM($V99:$AA99), 2),0)</f>
         <v/>
       </c>
@@ -13955,27 +13959,27 @@
       <c r="B100" s="26" t="n">
         <v>23</v>
       </c>
-      <c r="C100" s="54">
+      <c r="C100" s="41">
         <f>IF(SUM($V100:$AA100), ROUND(V100/SUM($V100:$AA100), 2),0)</f>
         <v/>
       </c>
-      <c r="D100" s="54">
+      <c r="D100" s="41">
         <f>IF(SUM($V100:$AA100), ROUND(W100/SUM($V100:$AA100), 2),0)</f>
         <v/>
       </c>
-      <c r="E100" s="54">
+      <c r="E100" s="41">
         <f>IF(SUM($V100:$AA100), ROUND(X100/SUM($V100:$AA100), 2),0)</f>
         <v/>
       </c>
-      <c r="F100" s="54">
+      <c r="F100" s="41">
         <f>IF(SUM($V100:$AA100), ROUND(Y100/SUM($V100:$AA100), 2),0)</f>
         <v/>
       </c>
-      <c r="G100" s="54">
+      <c r="G100" s="41">
         <f>IF(SUM($V100:$AA100), ROUND(Z100/SUM($V100:$AA100), 2),0)</f>
         <v/>
       </c>
-      <c r="H100" s="54">
+      <c r="H100" s="41">
         <f>IF(SUM($V100:$AA100), ROUND(AA100/SUM($V100:$AA100), 2),0)</f>
         <v/>
       </c>
@@ -14037,27 +14041,27 @@
       <c r="B101" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="C101" s="54">
+      <c r="C101" s="41">
         <f>IF(SUM($V101:$AA101), ROUND(V101/SUM($V101:$AA101), 2),0)</f>
         <v/>
       </c>
-      <c r="D101" s="54">
+      <c r="D101" s="41">
         <f>IF(SUM($V101:$AA101), ROUND(W101/SUM($V101:$AA101), 2),0)</f>
         <v/>
       </c>
-      <c r="E101" s="54">
+      <c r="E101" s="41">
         <f>IF(SUM($V101:$AA101), ROUND(X101/SUM($V101:$AA101), 2),0)</f>
         <v/>
       </c>
-      <c r="F101" s="54">
+      <c r="F101" s="41">
         <f>IF(SUM($V101:$AA101), ROUND(Y101/SUM($V101:$AA101), 2),0)</f>
         <v/>
       </c>
-      <c r="G101" s="54">
+      <c r="G101" s="41">
         <f>IF(SUM($V101:$AA101), ROUND(Z101/SUM($V101:$AA101), 2),0)</f>
         <v/>
       </c>
-      <c r="H101" s="54">
+      <c r="H101" s="41">
         <f>IF(SUM($V101:$AA101), ROUND(AA101/SUM($V101:$AA101), 2),0)</f>
         <v/>
       </c>
@@ -14119,27 +14123,27 @@
       <c r="B102" s="26" t="n">
         <v>34</v>
       </c>
-      <c r="C102" s="54">
+      <c r="C102" s="41">
         <f>IF(SUM($V102:$AA102), ROUND(V102/SUM($V102:$AA102), 2),0)</f>
         <v/>
       </c>
-      <c r="D102" s="54">
+      <c r="D102" s="41">
         <f>IF(SUM($V102:$AA102), ROUND(W102/SUM($V102:$AA102), 2),0)</f>
         <v/>
       </c>
-      <c r="E102" s="54">
+      <c r="E102" s="41">
         <f>IF(SUM($V102:$AA102), ROUND(X102/SUM($V102:$AA102), 2),0)</f>
         <v/>
       </c>
-      <c r="F102" s="54">
+      <c r="F102" s="41">
         <f>IF(SUM($V102:$AA102), ROUND(Y102/SUM($V102:$AA102), 2),0)</f>
         <v/>
       </c>
-      <c r="G102" s="54">
+      <c r="G102" s="41">
         <f>IF(SUM($V102:$AA102), ROUND(Z102/SUM($V102:$AA102), 2),0)</f>
         <v/>
       </c>
-      <c r="H102" s="54">
+      <c r="H102" s="41">
         <f>IF(SUM($V102:$AA102), ROUND(AA102/SUM($V102:$AA102), 2),0)</f>
         <v/>
       </c>
@@ -14201,27 +14205,27 @@
       <c r="B103" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="C103" s="54">
+      <c r="C103" s="41">
         <f>IF(SUM($V103:$AA103), ROUND(V103/SUM($V103:$AA103), 2),0)</f>
         <v/>
       </c>
-      <c r="D103" s="54">
+      <c r="D103" s="41">
         <f>IF(SUM($V103:$AA103), ROUND(W103/SUM($V103:$AA103), 2),0)</f>
         <v/>
       </c>
-      <c r="E103" s="54">
+      <c r="E103" s="41">
         <f>IF(SUM($V103:$AA103), ROUND(X103/SUM($V103:$AA103), 2),0)</f>
         <v/>
       </c>
-      <c r="F103" s="54">
+      <c r="F103" s="41">
         <f>IF(SUM($V103:$AA103), ROUND(Y103/SUM($V103:$AA103), 2),0)</f>
         <v/>
       </c>
-      <c r="G103" s="54">
+      <c r="G103" s="41">
         <f>IF(SUM($V103:$AA103), ROUND(Z103/SUM($V103:$AA103), 2),0)</f>
         <v/>
       </c>
-      <c r="H103" s="54">
+      <c r="H103" s="41">
         <f>IF(SUM($V103:$AA103), ROUND(AA103/SUM($V103:$AA103), 2),0)</f>
         <v/>
       </c>
@@ -14283,27 +14287,27 @@
       <c r="B104" s="26" t="n">
         <v>34</v>
       </c>
-      <c r="C104" s="54">
+      <c r="C104" s="41">
         <f>IF(SUM($V104:$AA104), ROUND(V104/SUM($V104:$AA104), 2),0)</f>
         <v/>
       </c>
-      <c r="D104" s="54">
+      <c r="D104" s="41">
         <f>IF(SUM($V104:$AA104), ROUND(W104/SUM($V104:$AA104), 2),0)</f>
         <v/>
       </c>
-      <c r="E104" s="54">
+      <c r="E104" s="41">
         <f>IF(SUM($V104:$AA104), ROUND(X104/SUM($V104:$AA104), 2),0)</f>
         <v/>
       </c>
-      <c r="F104" s="54">
+      <c r="F104" s="41">
         <f>IF(SUM($V104:$AA104), ROUND(Y104/SUM($V104:$AA104), 2),0)</f>
         <v/>
       </c>
-      <c r="G104" s="54">
+      <c r="G104" s="41">
         <f>IF(SUM($V104:$AA104), ROUND(Z104/SUM($V104:$AA104), 2),0)</f>
         <v/>
       </c>
-      <c r="H104" s="54">
+      <c r="H104" s="41">
         <f>IF(SUM($V104:$AA104), ROUND(AA104/SUM($V104:$AA104), 2),0)</f>
         <v/>
       </c>
@@ -14365,27 +14369,27 @@
       <c r="B105" s="26" t="n">
         <v>23</v>
       </c>
-      <c r="C105" s="54">
+      <c r="C105" s="41">
         <f>IF(SUM($V105:$AA105), ROUND(V105/SUM($V105:$AA105), 2),0)</f>
         <v/>
       </c>
-      <c r="D105" s="54">
+      <c r="D105" s="41">
         <f>IF(SUM($V105:$AA105), ROUND(W105/SUM($V105:$AA105), 2),0)</f>
         <v/>
       </c>
-      <c r="E105" s="54">
+      <c r="E105" s="41">
         <f>IF(SUM($V105:$AA105), ROUND(X105/SUM($V105:$AA105), 2),0)</f>
         <v/>
       </c>
-      <c r="F105" s="54">
+      <c r="F105" s="41">
         <f>IF(SUM($V105:$AA105), ROUND(Y105/SUM($V105:$AA105), 2),0)</f>
         <v/>
       </c>
-      <c r="G105" s="54">
+      <c r="G105" s="41">
         <f>IF(SUM($V105:$AA105), ROUND(Z105/SUM($V105:$AA105), 2),0)</f>
         <v/>
       </c>
-      <c r="H105" s="54">
+      <c r="H105" s="41">
         <f>IF(SUM($V105:$AA105), ROUND(AA105/SUM($V105:$AA105), 2),0)</f>
         <v/>
       </c>
@@ -14447,27 +14451,27 @@
       <c r="B106" s="26" t="n">
         <v>38</v>
       </c>
-      <c r="C106" s="54">
+      <c r="C106" s="41">
         <f>IF(SUM($V106:$AA106), ROUND(V106/SUM($V106:$AA106), 2),0)</f>
         <v/>
       </c>
-      <c r="D106" s="54">
+      <c r="D106" s="41">
         <f>IF(SUM($V106:$AA106), ROUND(W106/SUM($V106:$AA106), 2),0)</f>
         <v/>
       </c>
-      <c r="E106" s="54">
+      <c r="E106" s="41">
         <f>IF(SUM($V106:$AA106), ROUND(X106/SUM($V106:$AA106), 2),0)</f>
         <v/>
       </c>
-      <c r="F106" s="54">
+      <c r="F106" s="41">
         <f>IF(SUM($V106:$AA106), ROUND(Y106/SUM($V106:$AA106), 2),0)</f>
         <v/>
       </c>
-      <c r="G106" s="54">
+      <c r="G106" s="41">
         <f>IF(SUM($V106:$AA106), ROUND(Z106/SUM($V106:$AA106), 2),0)</f>
         <v/>
       </c>
-      <c r="H106" s="54">
+      <c r="H106" s="41">
         <f>IF(SUM($V106:$AA106), ROUND(AA106/SUM($V106:$AA106), 2),0)</f>
         <v/>
       </c>
@@ -14529,27 +14533,27 @@
       <c r="B107" s="26" t="n">
         <v>73</v>
       </c>
-      <c r="C107" s="54">
+      <c r="C107" s="41">
         <f>IF(SUM($V107:$AA107), ROUND(V107/SUM($V107:$AA107), 2),0)</f>
         <v/>
       </c>
-      <c r="D107" s="54">
+      <c r="D107" s="41">
         <f>IF(SUM($V107:$AA107), ROUND(W107/SUM($V107:$AA107), 2),0)</f>
         <v/>
       </c>
-      <c r="E107" s="54">
+      <c r="E107" s="41">
         <f>IF(SUM($V107:$AA107), ROUND(X107/SUM($V107:$AA107), 2),0)</f>
         <v/>
       </c>
-      <c r="F107" s="54">
+      <c r="F107" s="41">
         <f>IF(SUM($V107:$AA107), ROUND(Y107/SUM($V107:$AA107), 2),0)</f>
         <v/>
       </c>
-      <c r="G107" s="54">
+      <c r="G107" s="41">
         <f>IF(SUM($V107:$AA107), ROUND(Z107/SUM($V107:$AA107), 2),0)</f>
         <v/>
       </c>
-      <c r="H107" s="54">
+      <c r="H107" s="41">
         <f>IF(SUM($V107:$AA107), ROUND(AA107/SUM($V107:$AA107), 2),0)</f>
         <v/>
       </c>
@@ -14611,27 +14615,27 @@
       <c r="B108" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="C108" s="54">
+      <c r="C108" s="41">
         <f>IF(SUM($V108:$AA108), ROUND(V108/SUM($V108:$AA108), 2),0)</f>
         <v/>
       </c>
-      <c r="D108" s="54">
+      <c r="D108" s="41">
         <f>IF(SUM($V108:$AA108), ROUND(W108/SUM($V108:$AA108), 2),0)</f>
         <v/>
       </c>
-      <c r="E108" s="54">
+      <c r="E108" s="41">
         <f>IF(SUM($V108:$AA108), ROUND(X108/SUM($V108:$AA108), 2),0)</f>
         <v/>
       </c>
-      <c r="F108" s="54">
+      <c r="F108" s="41">
         <f>IF(SUM($V108:$AA108), ROUND(Y108/SUM($V108:$AA108), 2),0)</f>
         <v/>
       </c>
-      <c r="G108" s="54">
+      <c r="G108" s="41">
         <f>IF(SUM($V108:$AA108), ROUND(Z108/SUM($V108:$AA108), 2),0)</f>
         <v/>
       </c>
-      <c r="H108" s="54">
+      <c r="H108" s="41">
         <f>IF(SUM($V108:$AA108), ROUND(AA108/SUM($V108:$AA108), 2),0)</f>
         <v/>
       </c>
@@ -14693,27 +14697,27 @@
       <c r="B109" s="26" t="n">
         <v>21</v>
       </c>
-      <c r="C109" s="54">
+      <c r="C109" s="41">
         <f>IF(SUM($V109:$AA109), ROUND(V109/SUM($V109:$AA109), 2),0)</f>
         <v/>
       </c>
-      <c r="D109" s="54">
+      <c r="D109" s="41">
         <f>IF(SUM($V109:$AA109), ROUND(W109/SUM($V109:$AA109), 2),0)</f>
         <v/>
       </c>
-      <c r="E109" s="54">
+      <c r="E109" s="41">
         <f>IF(SUM($V109:$AA109), ROUND(X109/SUM($V109:$AA109), 2),0)</f>
         <v/>
       </c>
-      <c r="F109" s="54">
+      <c r="F109" s="41">
         <f>IF(SUM($V109:$AA109), ROUND(Y109/SUM($V109:$AA109), 2),0)</f>
         <v/>
       </c>
-      <c r="G109" s="54">
+      <c r="G109" s="41">
         <f>IF(SUM($V109:$AA109), ROUND(Z109/SUM($V109:$AA109), 2),0)</f>
         <v/>
       </c>
-      <c r="H109" s="54">
+      <c r="H109" s="41">
         <f>IF(SUM($V109:$AA109), ROUND(AA109/SUM($V109:$AA109), 2),0)</f>
         <v/>
       </c>
@@ -14775,27 +14779,27 @@
       <c r="B110" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C110" s="54">
+      <c r="C110" s="41">
         <f>IF(SUM($V110:$AA110), ROUND(V110/SUM($V110:$AA110), 2),0)</f>
         <v/>
       </c>
-      <c r="D110" s="54">
+      <c r="D110" s="41">
         <f>IF(SUM($V110:$AA110), ROUND(W110/SUM($V110:$AA110), 2),0)</f>
         <v/>
       </c>
-      <c r="E110" s="54">
+      <c r="E110" s="41">
         <f>IF(SUM($V110:$AA110), ROUND(X110/SUM($V110:$AA110), 2),0)</f>
         <v/>
       </c>
-      <c r="F110" s="54">
+      <c r="F110" s="41">
         <f>IF(SUM($V110:$AA110), ROUND(Y110/SUM($V110:$AA110), 2),0)</f>
         <v/>
       </c>
-      <c r="G110" s="54">
+      <c r="G110" s="41">
         <f>IF(SUM($V110:$AA110), ROUND(Z110/SUM($V110:$AA110), 2),0)</f>
         <v/>
       </c>
-      <c r="H110" s="54">
+      <c r="H110" s="41">
         <f>IF(SUM($V110:$AA110), ROUND(AA110/SUM($V110:$AA110), 2),0)</f>
         <v/>
       </c>
@@ -14857,27 +14861,27 @@
       <c r="B111" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="C111" s="54">
+      <c r="C111" s="41">
         <f>IF(SUM($V111:$AA111), ROUND(V111/SUM($V111:$AA111), 2),0)</f>
         <v/>
       </c>
-      <c r="D111" s="54">
+      <c r="D111" s="41">
         <f>IF(SUM($V111:$AA111), ROUND(W111/SUM($V111:$AA111), 2),0)</f>
         <v/>
       </c>
-      <c r="E111" s="54">
+      <c r="E111" s="41">
         <f>IF(SUM($V111:$AA111), ROUND(X111/SUM($V111:$AA111), 2),0)</f>
         <v/>
       </c>
-      <c r="F111" s="54">
+      <c r="F111" s="41">
         <f>IF(SUM($V111:$AA111), ROUND(Y111/SUM($V111:$AA111), 2),0)</f>
         <v/>
       </c>
-      <c r="G111" s="54">
+      <c r="G111" s="41">
         <f>IF(SUM($V111:$AA111), ROUND(Z111/SUM($V111:$AA111), 2),0)</f>
         <v/>
       </c>
-      <c r="H111" s="54">
+      <c r="H111" s="41">
         <f>IF(SUM($V111:$AA111), ROUND(AA111/SUM($V111:$AA111), 2),0)</f>
         <v/>
       </c>
@@ -14939,27 +14943,27 @@
       <c r="B112" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="C112" s="55">
+      <c r="C112" s="42">
         <f>IF(SUM($V112:$AA112), ROUND(V112/SUM($V112:$AA112), 2),0)</f>
         <v/>
       </c>
-      <c r="D112" s="55">
+      <c r="D112" s="42">
         <f>IF(SUM($V112:$AA112), ROUND(W112/SUM($V112:$AA112), 2),0)</f>
         <v/>
       </c>
-      <c r="E112" s="55">
+      <c r="E112" s="42">
         <f>IF(SUM($V112:$AA112), ROUND(X112/SUM($V112:$AA112), 2),0)</f>
         <v/>
       </c>
-      <c r="F112" s="55">
+      <c r="F112" s="42">
         <f>IF(SUM($V112:$AA112), ROUND(Y112/SUM($V112:$AA112), 2),0)</f>
         <v/>
       </c>
-      <c r="G112" s="55">
+      <c r="G112" s="42">
         <f>IF(SUM($V112:$AA112), ROUND(Z112/SUM($V112:$AA112), 2),0)</f>
         <v/>
       </c>
-      <c r="H112" s="55">
+      <c r="H112" s="42">
         <f>IF(SUM($V112:$AA112), ROUND(AA112/SUM($V112:$AA112), 2),0)</f>
         <v/>
       </c>
@@ -15394,16 +15398,13 @@
     <row r="123" ht="35.1" customHeight="1"/>
     <row r="124" ht="33.95" customHeight="1"/>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="9">
     <mergeCell ref="C11:H11"/>
-    <mergeCell ref="B6:C6"/>
     <mergeCell ref="V11:AA11"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B8:C8"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="O11:T11"/>
     <mergeCell ref="A11:A12"/>

</xml_diff>